<commit_message>
Att Dia 2 da Fase de 32
+ Correções de formatação dos classificados
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE93637-9C6E-434F-8D2E-067AEB248404}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF302D3-E586-40A4-B7C7-8C07227B9510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9525" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="7" r:id="rId1"/>
@@ -26,6 +26,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -2962,6 +2973,17 @@
     </dxf>
     <dxf>
       <font>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -3066,17 +3088,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -9037,25 +9048,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CB5EB0A-66D8-48B4-BC40-E2D214AFC03A}" name="Tabela1" displayName="Tabela1" ref="C3:E51" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CB5EB0A-66D8-48B4-BC40-E2D214AFC03A}" name="Tabela1" displayName="Tabela1" ref="C3:E51" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
   <autoFilter ref="C3:E51" xr:uid="{9CB5EB0A-66D8-48B4-BC40-E2D214AFC03A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{BA403FB9-D643-4201-89E9-82280DBD496D}" name=" " dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{8927B163-5C71-4390-8413-1CB7AFCDC479}" name="Times" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{95E8A229-CD3E-4FE0-BC0B-3E68BBDC2143}" name="  " dataDxfId="84"/>
+    <tableColumn id="1" xr3:uid="{BA403FB9-D643-4201-89E9-82280DBD496D}" name=" " dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{8927B163-5C71-4390-8413-1CB7AFCDC479}" name="Times" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{95E8A229-CD3E-4FE0-BC0B-3E68BBDC2143}" name="  " dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -9093,7 +9104,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -9199,7 +9210,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -9341,7 +9352,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9650,12 +9661,12 @@
     <mergeCell ref="J33:L33"/>
   </mergeCells>
   <conditionalFormatting sqref="J31:L31 J32:J33">
-    <cfRule type="cellIs" dxfId="90" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="2" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J31:L33">
-    <cfRule type="expression" dxfId="89" priority="1">
+    <cfRule type="expression" dxfId="84" priority="1">
       <formula>M31&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22079,7 +22090,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="yMneGrh/V9v9I71ExvSu/Y2aQsnzReoZXlElqaiRdEFQ/HU0DofiNVmtRyr1uLMjGEnHu5TZOHdJIGeVyKwyVA==" saltValue="Bgw7AbWnF5ZQuHYiR+WIGA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="jYYlVwSGK2cwUbCoz9yiV/3/qarQWCd0N5s5n0ASO0lHveA2ehdpEX2q+Q+OAp4tWRG8yzgngnOerW0AMWPDhQ==" saltValue="7vEdaL9dS3g/pLdxzX+azg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="1">
     <mergeCell ref="F3:H3"/>
   </mergeCells>
@@ -22163,7 +22174,7 @@
       <formula>AH6=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF12:AF13 AF18:AF19 AF24:AF25 AF30:AF31 AF36:AF37 AF42:AF43 AF48:AF49 AF60:AF61 AF66:AF67 AF72:AF73 AF54:AF55">
+  <conditionalFormatting sqref="AF12:AF13 AF18:AF19 AF24:AF25 AF30:AF31 AF36:AF37 AF42:AF43 AF48:AF49 AF54:AF55 AF60:AF61 AF66:AF67 AF72:AF73">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>AH12=3</formula>
     </cfRule>
@@ -22178,7 +22189,7 @@
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BJ6:BJ13">
+  <conditionalFormatting sqref="BJ6:BJ17">
     <cfRule type="expression" dxfId="0" priority="77">
       <formula>BL6=3</formula>
     </cfRule>
@@ -54668,11 +54679,15 @@
         <v>África do Sul</v>
       </c>
       <c r="F5" s="149"/>
-      <c r="G5" s="123"/>
+      <c r="G5" s="123">
+        <v>0</v>
+      </c>
       <c r="H5" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="123"/>
+      <c r="I5" s="123">
+        <v>1</v>
+      </c>
       <c r="J5" s="150"/>
       <c r="K5" s="151" t="str">
         <f>IF('Fase de Grupos'!AH13=3,'Fase de Grupos'!AF13,"2º do Grupo B")</f>
@@ -54684,7 +54699,7 @@
       </c>
       <c r="M5" s="133" t="str">
         <f>IF(OR(G5="",I5=""),"Vencedor 73",IF(G5&lt;&gt;I5,IF(G5&gt;I5,E5,K5),IF(SUM(F5:G5)=SUM(I5:J5),"Vencedor 73",IF(SUM(F5:G5)&gt;SUM(I5:J5),E5,K5))))</f>
-        <v>Vencedor 73</v>
+        <v>Canadá</v>
       </c>
       <c r="N5" s="133">
         <v>73</v>
@@ -54741,24 +54756,32 @@
         <f>IF('Fase de Grupos'!AH30=3,'Fase de Grupos'!AF30,"1º do Grupo E")</f>
         <v>Alemanha</v>
       </c>
-      <c r="F6" s="149"/>
-      <c r="G6" s="123"/>
+      <c r="F6" s="149">
+        <v>3</v>
+      </c>
+      <c r="G6" s="123">
+        <v>1</v>
+      </c>
       <c r="H6" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I6" s="123"/>
-      <c r="J6" s="150"/>
+      <c r="I6" s="123">
+        <v>1</v>
+      </c>
+      <c r="J6" s="150">
+        <v>4</v>
+      </c>
       <c r="K6" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R11,"3º A, B, C, D ou F")</f>
         <v>Paraguai</v>
       </c>
       <c r="L6" s="136" t="str">
         <f t="shared" ref="L6:L12" si="0">IF(OR(G6="",I6=""),"",IF(G6=I6,"emp",""))</f>
-        <v/>
+        <v>emp</v>
       </c>
       <c r="M6" s="133" t="str">
         <f>IF(OR(G6="",I6=""),"Vencedor 74",IF(G6&lt;&gt;I6,IF(G6&gt;I6,E6,K6),IF(SUM(F6:G6)=SUM(I6:J6),"Vencedor 74",IF(SUM(F6:G6)&gt;SUM(I6:J6),E6,K6))))</f>
-        <v>Vencedor 74</v>
+        <v>Paraguai</v>
       </c>
       <c r="N6" s="133">
         <v>74</v>
@@ -54819,24 +54842,32 @@
         <f>IF('Fase de Grupos'!AH36=3,'Fase de Grupos'!AF36,"1º do Grupo F")</f>
         <v>Países Baixos</v>
       </c>
-      <c r="F7" s="149"/>
-      <c r="G7" s="123"/>
+      <c r="F7" s="149">
+        <v>2</v>
+      </c>
+      <c r="G7" s="123">
+        <v>1</v>
+      </c>
       <c r="H7" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="123"/>
-      <c r="J7" s="150"/>
+      <c r="I7" s="123">
+        <v>1</v>
+      </c>
+      <c r="J7" s="150">
+        <v>3</v>
+      </c>
       <c r="K7" s="151" t="str">
         <f>IF('Fase de Grupos'!AH19=3,'Fase de Grupos'!AF19,"2º do Grupo C")</f>
         <v>Marrocos</v>
       </c>
       <c r="L7" s="136" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>emp</v>
       </c>
       <c r="M7" s="133" t="str">
         <f>IF(OR(G7="",I7=""),"Vencedor 75",IF(G7&lt;&gt;I7,IF(G7&gt;I7,E7,K7),IF(SUM(F7:G7)=SUM(I7:J7),"Vencedor 75",IF(SUM(F7:G7)&gt;SUM(I7:J7),E7,K7))))</f>
-        <v>Vencedor 75</v>
+        <v>Marrocos</v>
       </c>
       <c r="N7" s="133">
         <v>75</v>
@@ -54894,11 +54925,15 @@
         <v>Brasil</v>
       </c>
       <c r="F8" s="149"/>
-      <c r="G8" s="123"/>
+      <c r="G8" s="123">
+        <v>2</v>
+      </c>
       <c r="H8" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="123"/>
+      <c r="I8" s="123">
+        <v>1</v>
+      </c>
       <c r="J8" s="150"/>
       <c r="K8" s="151" t="str">
         <f>IF('Fase de Grupos'!AH37=3,'Fase de Grupos'!AF37,"2º do Grupo F")</f>
@@ -54910,7 +54945,7 @@
       </c>
       <c r="M8" s="133" t="str">
         <f>IF(OR(G8="",I8=""),"Vencedor 76",IF(G8&lt;&gt;I8,IF(G8&gt;I8,E8,K8),IF(SUM(F8:G8)=SUM(I8:J8),"Vencedor 76",IF(SUM(F8:G8)&gt;SUM(I8:J8),E8,K8))))</f>
-        <v>Vencedor 76</v>
+        <v>Brasil</v>
       </c>
       <c r="N8" s="133">
         <v>76</v>
@@ -56029,7 +56064,7 @@
       </c>
       <c r="E25" s="106" t="str">
         <f>M6</f>
-        <v>Vencedor 74</v>
+        <v>Paraguai</v>
       </c>
       <c r="F25" s="149"/>
       <c r="G25" s="123"/>
@@ -56107,7 +56142,7 @@
       </c>
       <c r="E26" s="106" t="str">
         <f>M5</f>
-        <v>Vencedor 73</v>
+        <v>Canadá</v>
       </c>
       <c r="F26" s="149"/>
       <c r="G26" s="123"/>
@@ -56118,7 +56153,7 @@
       <c r="J26" s="150"/>
       <c r="K26" s="151" t="str">
         <f>M7</f>
-        <v>Vencedor 75</v>
+        <v>Marrocos</v>
       </c>
       <c r="L26" s="136" t="str">
         <f t="shared" ref="L26:L32" si="18">IF(OR(G26="",I26=""),"",IF(G26=I26,"emp",""))</f>
@@ -56151,7 +56186,7 @@
       </c>
       <c r="E27" s="106" t="str">
         <f>M8</f>
-        <v>Vencedor 76</v>
+        <v>Brasil</v>
       </c>
       <c r="F27" s="149"/>
       <c r="G27" s="123"/>
@@ -57403,7 +57438,7 @@
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="c6tPJJQuMaLYYVxDkvgugaxcC+Uv5gkJkUqZgIt2uuxbzexMxqxVyEOkWorUUitpEJ1MPNBlUf/aYq65/wymIg==" saltValue="0J8NZQ0DnJYkRWhoKBlPHA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
-  <sortState ref="C59:C64">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C59:C64">
     <sortCondition ref="C59:C64"/>
   </sortState>
   <mergeCells count="16">

</xml_diff>

<commit_message>
Att Dia 3 da Fase de 32
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF302D3-E586-40A4-B7C7-8C07227B9510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D0651F-0D3B-4A43-AD72-F33B298C78AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
@@ -2178,123 +2178,6 @@
   </cellStyles>
   <dxfs count="91">
     <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
@@ -2742,6 +2625,123 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -22095,102 +22095,102 @@
     <mergeCell ref="F3:H3"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A51 P3 B3:O51">
-    <cfRule type="cellIs" dxfId="19" priority="215" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="215" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A52:O75">
-    <cfRule type="cellIs" dxfId="18" priority="136" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="136" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:E9">
-    <cfRule type="cellIs" dxfId="17" priority="202" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="202" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:E21">
-    <cfRule type="cellIs" dxfId="16" priority="193" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="193" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:E33">
-    <cfRule type="cellIs" dxfId="15" priority="191" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="191" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C40:E45">
-    <cfRule type="cellIs" dxfId="14" priority="189" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="189" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C52:E57">
-    <cfRule type="cellIs" dxfId="13" priority="130" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="130" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C64:E69">
-    <cfRule type="cellIs" dxfId="12" priority="128" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="128" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:I9">
-    <cfRule type="cellIs" dxfId="11" priority="198" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="198" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16:I21">
-    <cfRule type="cellIs" dxfId="10" priority="188" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="188" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I28:I33">
-    <cfRule type="cellIs" dxfId="9" priority="187" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="187" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I40:I45">
-    <cfRule type="cellIs" dxfId="8" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="186" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I52:I57">
-    <cfRule type="cellIs" dxfId="7" priority="127" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="127" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I64:I69">
-    <cfRule type="cellIs" dxfId="6" priority="126" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="126" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:AN75">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6:AF7">
-    <cfRule type="expression" dxfId="4" priority="209">
+    <cfRule type="expression" dxfId="32" priority="209">
       <formula>AH6=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF12:AF13 AF18:AF19 AF24:AF25 AF30:AF31 AF36:AF37 AF42:AF43 AF48:AF49 AF54:AF55 AF60:AF61 AF66:AF67 AF72:AF73">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="31" priority="1">
       <formula>AH12=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AP5:BG17">
-    <cfRule type="cellIs" dxfId="2" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="83" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BI4:BR17">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="2" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BJ6:BJ17">
-    <cfRule type="expression" dxfId="0" priority="77">
+    <cfRule type="expression" dxfId="28" priority="77">
       <formula>BL6=3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -55020,11 +55020,15 @@
         <v>França</v>
       </c>
       <c r="F9" s="149"/>
-      <c r="G9" s="123"/>
+      <c r="G9" s="123">
+        <v>3</v>
+      </c>
       <c r="H9" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="123"/>
+      <c r="I9" s="123">
+        <v>0</v>
+      </c>
       <c r="J9" s="150"/>
       <c r="K9" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R13,"3º C, D, F, G ou H")</f>
@@ -55036,7 +55040,7 @@
       </c>
       <c r="M9" s="133" t="str">
         <f>IF(OR(G9="",I9=""),"Vencedor 77",IF(G9&lt;&gt;I9,IF(G9&gt;I9,E9,K9),IF(SUM(F9:G9)=SUM(I9:J9),"Vencedor 77",IF(SUM(F9:G9)&gt;SUM(I9:J9),E9,K9))))</f>
-        <v>Vencedor 77</v>
+        <v>França</v>
       </c>
       <c r="N9" s="133">
         <v>77</v>
@@ -55092,11 +55096,15 @@
         <v>Costa do Marfim</v>
       </c>
       <c r="F10" s="149"/>
-      <c r="G10" s="123"/>
+      <c r="G10" s="123">
+        <v>1</v>
+      </c>
       <c r="H10" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I10" s="123"/>
+      <c r="I10" s="123">
+        <v>2</v>
+      </c>
       <c r="J10" s="150"/>
       <c r="K10" s="151" t="str">
         <f>IF('Fase de Grupos'!AH55=3,'Fase de Grupos'!AF55,"2º do Grupo I")</f>
@@ -55108,7 +55116,7 @@
       </c>
       <c r="M10" s="133" t="str">
         <f>IF(OR(G10="",I10=""),"Vencedor 78",IF(G10&lt;&gt;I10,IF(G10&gt;I10,E10,K10),IF(SUM(F10:G10)=SUM(I10:J10),"Vencedor 78",IF(SUM(F10:G10)&gt;SUM(I10:J10),E10,K10))))</f>
-        <v>Vencedor 78</v>
+        <v>Noruega</v>
       </c>
       <c r="N10" s="133">
         <v>78</v>
@@ -55164,11 +55172,15 @@
         <v>México</v>
       </c>
       <c r="F11" s="149"/>
-      <c r="G11" s="123"/>
+      <c r="G11" s="123">
+        <v>2</v>
+      </c>
       <c r="H11" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="123"/>
+      <c r="I11" s="123">
+        <v>0</v>
+      </c>
       <c r="J11" s="150"/>
       <c r="K11" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R8,"3º C, E, F, H ou I")</f>
@@ -55180,7 +55192,7 @@
       </c>
       <c r="M11" s="133" t="str">
         <f>IF(OR(G11="",I11=""),"Vencedor 79",IF(G11&lt;&gt;I11,IF(G11&gt;I11,E11,K11),IF(SUM(F11:G11)=SUM(I11:J11),"Vencedor 79",IF(SUM(F11:G11)&gt;SUM(I11:J11),E11,K11))))</f>
-        <v>Vencedor 79</v>
+        <v>México</v>
       </c>
       <c r="N11" s="133">
         <v>79</v>
@@ -56075,7 +56087,7 @@
       <c r="J25" s="150"/>
       <c r="K25" s="151" t="str">
         <f>M9</f>
-        <v>Vencedor 77</v>
+        <v>França</v>
       </c>
       <c r="L25" s="136" t="str">
         <f>IF(OR(G25="",I25=""),"",IF(G25=I25,"emp",""))</f>
@@ -56197,7 +56209,7 @@
       <c r="J27" s="150"/>
       <c r="K27" s="151" t="str">
         <f>M10</f>
-        <v>Vencedor 78</v>
+        <v>Noruega</v>
       </c>
       <c r="L27" s="136" t="str">
         <f t="shared" si="18"/>
@@ -56230,7 +56242,7 @@
       </c>
       <c r="E28" s="106" t="str">
         <f>M11</f>
-        <v>Vencedor 79</v>
+        <v>México</v>
       </c>
       <c r="F28" s="149"/>
       <c r="G28" s="123"/>
@@ -56682,142 +56694,142 @@
     <mergeCell ref="Y34:AA34"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A2 B2:K2 X9:AG10 X15:AG16 X20:AG21 B21:K22 AB34:AB36 A57:K58 H59:K61 B62:K71 B83:K1048576">
-    <cfRule type="cellIs" dxfId="47" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="76" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:B12 C4:K12">
-    <cfRule type="cellIs" dxfId="46" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="42" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13:K20">
-    <cfRule type="cellIs" dxfId="45" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="31" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B36 C24:K33">
-    <cfRule type="cellIs" dxfId="44" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="20" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F20">
-    <cfRule type="expression" dxfId="43" priority="30">
+    <cfRule type="expression" dxfId="23" priority="30">
       <formula>L5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F25:F32">
-    <cfRule type="expression" dxfId="42" priority="19">
+    <cfRule type="expression" dxfId="22" priority="19">
       <formula>L25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J20">
-    <cfRule type="expression" dxfId="41" priority="29">
+    <cfRule type="expression" dxfId="21" priority="29">
       <formula>L5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J25:J32">
-    <cfRule type="expression" dxfId="40" priority="18">
+    <cfRule type="expression" dxfId="20" priority="18">
       <formula>L25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K20">
-    <cfRule type="expression" dxfId="39" priority="21">
+    <cfRule type="expression" dxfId="19" priority="21">
       <formula>Q5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25:K32">
-    <cfRule type="expression" dxfId="38" priority="17">
+    <cfRule type="expression" dxfId="18" priority="17">
       <formula>Q25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W3:W24 A21:A34 I34:K34 Y34:AB34 Y34:Y36 A62:A1048576">
-    <cfRule type="cellIs" dxfId="37" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="77" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X3:X8 Y4:AG8">
-    <cfRule type="cellIs" dxfId="36" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="16" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X11:X14 Y12:AG14">
-    <cfRule type="cellIs" dxfId="35" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="12" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X17:X19 Y18:AG19">
-    <cfRule type="cellIs" dxfId="34" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="8" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X23:X25 Y24:AG25">
-    <cfRule type="cellIs" dxfId="33" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="4" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y34:AA36">
-    <cfRule type="expression" dxfId="32" priority="65">
+    <cfRule type="expression" dxfId="12" priority="65">
       <formula>AB34&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB5:AB8">
-    <cfRule type="expression" dxfId="31" priority="15">
+    <cfRule type="expression" dxfId="11" priority="15">
       <formula>AH5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB13:AB14">
-    <cfRule type="expression" dxfId="30" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>AH13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB19">
-    <cfRule type="expression" dxfId="29" priority="7">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AH19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB25">
-    <cfRule type="expression" dxfId="28" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>AH25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AF8">
-    <cfRule type="expression" dxfId="27" priority="14">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>AH5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF13:AF14">
-    <cfRule type="expression" dxfId="26" priority="10">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>AH13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF19">
-    <cfRule type="expression" dxfId="25" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>AH19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF25">
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>AH25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG5:AG8">
-    <cfRule type="expression" dxfId="23" priority="13">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>AM5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG13:AG14">
-    <cfRule type="expression" dxfId="22" priority="9">
+    <cfRule type="expression" dxfId="2" priority="9">
       <formula>AM13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG19">
-    <cfRule type="expression" dxfId="21" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>AM19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG25">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>AM25="emp"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Correções formatação dos classificados
+ Apoio
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D0651F-0D3B-4A43-AD72-F33B298C78AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9699A2C-6FD9-466F-82D7-B46D28F5B04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8985" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8987" uniqueCount="212">
   <si>
     <t>Times</t>
   </si>
@@ -786,6 +786,9 @@
       <t>.</t>
     </r>
   </si>
+  <si>
+    <t>Apoio</t>
+  </si>
 </sst>
 </file>
 
@@ -1125,7 +1128,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -1643,12 +1646,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="211">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2138,6 +2161,15 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2148,15 +2180,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2171,12 +2194,142 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="91">
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2625,123 +2778,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -5114,6 +5150,178 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>4763</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>766762</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95419BAC-1011-4E09-ADE6-2668E33B6843}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
+              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a14:imgLayer r:embed="rId5">
+                  <a14:imgEffect>
+                    <a14:colorTemperature colorTemp="4700"/>
+                  </a14:imgEffect>
+                </a14:imgLayer>
+              </a14:imgProps>
+            </a:ext>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8501063" y="5429250"/>
+          <a:ext cx="761999" cy="761999"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>769145</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>64</xdr:col>
+      <xdr:colOff>245270</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>188119</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="CaixaDeTexto 3">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6588783-5929-4477-B6BE-15E2394DA1B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10646570" y="4343400"/>
+          <a:ext cx="1352550" cy="759619"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Rei da Pechincha</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="pt-BR" sz="800" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Promoções &amp;</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> Achadinhos</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5168,6 +5376,178 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>4763</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>223837</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagem 3">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5AEEA6ED-56F8-5305-26CE-2D6B3691CE3E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
+              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a14:imgLayer r:embed="rId5">
+                  <a14:imgEffect>
+                    <a14:colorTemperature colorTemp="4700"/>
+                  </a14:imgEffect>
+                </a14:imgLayer>
+              </a14:imgProps>
+            </a:ext>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8501063" y="5429250"/>
+          <a:ext cx="761999" cy="761999"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>226220</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>1378744</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>188119</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="CaixaDeTexto 4">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{230368B4-4B95-1780-08EC-C6FAD6D525D1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9265445" y="5429250"/>
+          <a:ext cx="1152524" cy="759619"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Rei da Pechincha</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="pt-BR" sz="800" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Promoções &amp;</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> Achadinhos</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Albertus MT Lt" panose="020E0502030304020304" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -9654,7 +10034,7 @@
       <c r="L33" s="183"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="R7MKfGIr3q3KasSJACKADhTt/LYOodNa9tmtKJjgNCMenwB8F4JksD1Wb6Inyd7c0WaCL2TG1h5loB5f76zIiQ==" saltValue="vzSxU7R4LDF7bDaBkhG3gA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="JhGV6VcDyvc3i9om8xFJD2TTjYS4KxdyrPHqfmvoUHY8jTzdLhnXdEDqhfq9o8QSGpM59e0FFua65Es5mRgoOA==" saltValue="uIq4f/wxSDvjcYmJtVUiRQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="J31:L31"/>
     <mergeCell ref="J32:L32"/>
@@ -14992,6 +15372,12 @@
         <f t="shared" ref="AR22:AR28" si="37">CODE(AQ22)</f>
         <v>70</v>
       </c>
+      <c r="BJ22" s="193" t="s">
+        <v>211</v>
+      </c>
+      <c r="BK22" s="194"/>
+      <c r="BL22" s="194"/>
+      <c r="BM22" s="195"/>
     </row>
     <row r="23" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A23" s="45"/>
@@ -15125,6 +15511,10 @@
         <f t="shared" si="37"/>
         <v>69</v>
       </c>
+      <c r="BJ23" s="205"/>
+      <c r="BK23" s="204"/>
+      <c r="BL23" s="204"/>
+      <c r="BM23" s="206"/>
     </row>
     <row r="24" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A24" s="45"/>
@@ -15281,6 +15671,10 @@
         <f t="shared" si="37"/>
         <v>76</v>
       </c>
+      <c r="BJ24" s="205"/>
+      <c r="BK24" s="204"/>
+      <c r="BL24" s="204"/>
+      <c r="BM24" s="207"/>
     </row>
     <row r="25" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A25" s="45"/>
@@ -15437,6 +15831,10 @@
         <f t="shared" si="37"/>
         <v>66</v>
       </c>
+      <c r="BJ25" s="205"/>
+      <c r="BK25" s="204"/>
+      <c r="BL25" s="204"/>
+      <c r="BM25" s="207"/>
     </row>
     <row r="26" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A26" s="45"/>
@@ -15593,6 +15991,10 @@
         <f t="shared" si="37"/>
         <v>74</v>
       </c>
+      <c r="BJ26" s="208"/>
+      <c r="BK26" s="209"/>
+      <c r="BL26" s="209"/>
+      <c r="BM26" s="210"/>
     </row>
     <row r="27" spans="1:70" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="45"/>
@@ -22090,107 +22492,108 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="jYYlVwSGK2cwUbCoz9yiV/3/qarQWCd0N5s5n0ASO0lHveA2ehdpEX2q+Q+OAp4tWRG8yzgngnOerW0AMWPDhQ==" saltValue="7vEdaL9dS3g/pLdxzX+azg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
-  <mergeCells count="1">
+  <sheetProtection algorithmName="SHA-512" hashValue="8zT4037DyHXrLqdq5iYyYrMR0TWaotldz5hVI4fTDbdqZ7l+Cxdqs/9/FGMP4061jLNiKfePtLYXoWPo6TdRXA==" saltValue="fkE/EIHEl7y+xiKxPcgv5w==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <mergeCells count="2">
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="BJ22:BM22"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A51 P3 B3:O51">
-    <cfRule type="cellIs" dxfId="47" priority="215" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="215" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A52:O75">
-    <cfRule type="cellIs" dxfId="46" priority="136" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="136" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:E9">
-    <cfRule type="cellIs" dxfId="45" priority="202" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="202" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:E21">
-    <cfRule type="cellIs" dxfId="44" priority="193" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="193" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:E33">
-    <cfRule type="cellIs" dxfId="43" priority="191" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="191" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C40:E45">
-    <cfRule type="cellIs" dxfId="42" priority="189" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="189" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C52:E57">
-    <cfRule type="cellIs" dxfId="41" priority="130" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="130" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C64:E69">
-    <cfRule type="cellIs" dxfId="40" priority="128" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="128" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:I9">
-    <cfRule type="cellIs" dxfId="39" priority="198" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="198" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16:I21">
-    <cfRule type="cellIs" dxfId="38" priority="188" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="188" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I28:I33">
-    <cfRule type="cellIs" dxfId="37" priority="187" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="187" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I40:I45">
-    <cfRule type="cellIs" dxfId="36" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="186" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I52:I57">
-    <cfRule type="cellIs" dxfId="35" priority="127" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="127" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I64:I69">
-    <cfRule type="cellIs" dxfId="34" priority="126" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="126" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:AN75">
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6:AF7">
-    <cfRule type="expression" dxfId="32" priority="209">
+    <cfRule type="expression" dxfId="4" priority="209">
       <formula>AH6=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF12:AF13 AF18:AF19 AF24:AF25 AF30:AF31 AF36:AF37 AF42:AF43 AF48:AF49 AF54:AF55 AF60:AF61 AF66:AF67 AF72:AF73">
-    <cfRule type="expression" dxfId="31" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>AH12=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AP5:BG17">
-    <cfRule type="cellIs" dxfId="30" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="83" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BI4:BR17">
-    <cfRule type="cellIs" dxfId="29" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BJ6:BJ17">
-    <cfRule type="expression" dxfId="28" priority="77">
+  <conditionalFormatting sqref="BJ6:BJ13">
+    <cfRule type="expression" dxfId="0" priority="77">
       <formula>BL6=3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -54570,18 +54973,18 @@
     </row>
     <row r="3" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A3" s="130"/>
-      <c r="B3" s="197" t="s">
+      <c r="B3" s="193" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="198"/>
-      <c r="D3" s="198"/>
-      <c r="E3" s="198"/>
-      <c r="F3" s="198"/>
-      <c r="G3" s="198"/>
-      <c r="H3" s="198"/>
-      <c r="I3" s="198"/>
-      <c r="J3" s="198"/>
-      <c r="K3" s="199"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="194"/>
+      <c r="F3" s="194"/>
+      <c r="G3" s="194"/>
+      <c r="H3" s="194"/>
+      <c r="I3" s="194"/>
+      <c r="J3" s="194"/>
+      <c r="K3" s="195"/>
       <c r="L3" s="131"/>
       <c r="M3" s="132"/>
       <c r="N3" s="132"/>
@@ -54589,18 +54992,18 @@
       <c r="P3" s="132"/>
       <c r="Q3" s="132"/>
       <c r="W3" s="130"/>
-      <c r="X3" s="197" t="s">
+      <c r="X3" s="193" t="s">
         <v>73</v>
       </c>
-      <c r="Y3" s="198"/>
-      <c r="Z3" s="198"/>
-      <c r="AA3" s="198"/>
-      <c r="AB3" s="198"/>
-      <c r="AC3" s="198"/>
-      <c r="AD3" s="198"/>
-      <c r="AE3" s="198"/>
-      <c r="AF3" s="198"/>
-      <c r="AG3" s="199"/>
+      <c r="Y3" s="194"/>
+      <c r="Z3" s="194"/>
+      <c r="AA3" s="194"/>
+      <c r="AB3" s="194"/>
+      <c r="AC3" s="194"/>
+      <c r="AD3" s="194"/>
+      <c r="AE3" s="194"/>
+      <c r="AF3" s="194"/>
+      <c r="AG3" s="195"/>
       <c r="AH3" s="131"/>
       <c r="AI3" s="132"/>
       <c r="AJ3" s="132"/>
@@ -54617,19 +55020,19 @@
       <c r="D4" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="193" t="s">
+      <c r="E4" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="193"/>
-      <c r="G4" s="193" t="s">
+      <c r="F4" s="196"/>
+      <c r="G4" s="196" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="193"/>
-      <c r="I4" s="193"/>
-      <c r="J4" s="193" t="s">
+      <c r="H4" s="196"/>
+      <c r="I4" s="196"/>
+      <c r="J4" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="193"/>
+      <c r="K4" s="196"/>
       <c r="L4" s="135"/>
       <c r="M4" s="135"/>
       <c r="N4" s="135"/>
@@ -54644,19 +55047,19 @@
       <c r="Z4" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="193" t="s">
+      <c r="AA4" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AB4" s="193"/>
-      <c r="AC4" s="193" t="s">
+      <c r="AB4" s="196"/>
+      <c r="AC4" s="196" t="s">
         <v>18</v>
       </c>
-      <c r="AD4" s="193"/>
-      <c r="AE4" s="193"/>
-      <c r="AF4" s="193" t="s">
+      <c r="AD4" s="196"/>
+      <c r="AE4" s="196"/>
+      <c r="AF4" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AG4" s="193"/>
+      <c r="AG4" s="196"/>
       <c r="AH4" s="136"/>
       <c r="AI4" s="133"/>
       <c r="AJ4" s="133"/>
@@ -55216,18 +55619,18 @@
         <v>12</v>
       </c>
       <c r="W11" s="130"/>
-      <c r="X11" s="197" t="s">
+      <c r="X11" s="193" t="s">
         <v>74</v>
       </c>
-      <c r="Y11" s="198"/>
-      <c r="Z11" s="198"/>
-      <c r="AA11" s="198"/>
-      <c r="AB11" s="198"/>
-      <c r="AC11" s="198"/>
-      <c r="AD11" s="198"/>
-      <c r="AE11" s="198"/>
-      <c r="AF11" s="198"/>
-      <c r="AG11" s="199"/>
+      <c r="Y11" s="194"/>
+      <c r="Z11" s="194"/>
+      <c r="AA11" s="194"/>
+      <c r="AB11" s="194"/>
+      <c r="AC11" s="194"/>
+      <c r="AD11" s="194"/>
+      <c r="AE11" s="194"/>
+      <c r="AF11" s="194"/>
+      <c r="AG11" s="195"/>
       <c r="AH11" s="131"/>
       <c r="AI11" s="132"/>
       <c r="AJ11" s="132"/>
@@ -55297,19 +55700,19 @@
       <c r="Z12" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA12" s="193" t="s">
+      <c r="AA12" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AB12" s="193"/>
-      <c r="AC12" s="193" t="s">
+      <c r="AB12" s="196"/>
+      <c r="AC12" s="196" t="s">
         <v>18</v>
       </c>
-      <c r="AD12" s="193"/>
-      <c r="AE12" s="193"/>
-      <c r="AF12" s="193" t="s">
+      <c r="AD12" s="196"/>
+      <c r="AE12" s="196"/>
+      <c r="AF12" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AG12" s="193"/>
+      <c r="AG12" s="196"/>
       <c r="AH12" s="136"/>
       <c r="AI12" s="133"/>
       <c r="AJ12" s="133"/>
@@ -55684,18 +56087,18 @@
         <v>30</v>
       </c>
       <c r="W17" s="130"/>
-      <c r="X17" s="197" t="s">
+      <c r="X17" s="193" t="s">
         <v>77</v>
       </c>
-      <c r="Y17" s="198"/>
-      <c r="Z17" s="198"/>
-      <c r="AA17" s="198"/>
-      <c r="AB17" s="198"/>
-      <c r="AC17" s="198"/>
-      <c r="AD17" s="198"/>
-      <c r="AE17" s="198"/>
-      <c r="AF17" s="198"/>
-      <c r="AG17" s="199"/>
+      <c r="Y17" s="194"/>
+      <c r="Z17" s="194"/>
+      <c r="AA17" s="194"/>
+      <c r="AB17" s="194"/>
+      <c r="AC17" s="194"/>
+      <c r="AD17" s="194"/>
+      <c r="AE17" s="194"/>
+      <c r="AF17" s="194"/>
+      <c r="AG17" s="195"/>
       <c r="AH17" s="131"/>
       <c r="AI17" s="132"/>
       <c r="AJ17" s="132"/>
@@ -55754,19 +56157,19 @@
       <c r="Z18" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA18" s="193" t="s">
+      <c r="AA18" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AB18" s="193"/>
-      <c r="AC18" s="193" t="s">
+      <c r="AB18" s="196"/>
+      <c r="AC18" s="196" t="s">
         <v>18</v>
       </c>
-      <c r="AD18" s="193"/>
-      <c r="AE18" s="193"/>
-      <c r="AF18" s="193" t="s">
+      <c r="AD18" s="196"/>
+      <c r="AE18" s="196"/>
+      <c r="AF18" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AG18" s="193"/>
+      <c r="AG18" s="196"/>
       <c r="AH18" s="136"/>
       <c r="AI18" s="133"/>
       <c r="AJ18" s="133"/>
@@ -55958,18 +56361,18 @@
     </row>
     <row r="23" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A23" s="130"/>
-      <c r="B23" s="197" t="s">
+      <c r="B23" s="193" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="198"/>
-      <c r="D23" s="198"/>
-      <c r="E23" s="198"/>
-      <c r="F23" s="198"/>
-      <c r="G23" s="198"/>
-      <c r="H23" s="198"/>
-      <c r="I23" s="198"/>
-      <c r="J23" s="198"/>
-      <c r="K23" s="199"/>
+      <c r="C23" s="194"/>
+      <c r="D23" s="194"/>
+      <c r="E23" s="194"/>
+      <c r="F23" s="194"/>
+      <c r="G23" s="194"/>
+      <c r="H23" s="194"/>
+      <c r="I23" s="194"/>
+      <c r="J23" s="194"/>
+      <c r="K23" s="195"/>
       <c r="L23" s="131"/>
       <c r="M23" s="132"/>
       <c r="N23" s="132"/>
@@ -55984,18 +56387,18 @@
         <v>48</v>
       </c>
       <c r="W23" s="45"/>
-      <c r="X23" s="197" t="s">
+      <c r="X23" s="193" t="s">
         <v>79</v>
       </c>
-      <c r="Y23" s="198"/>
-      <c r="Z23" s="198"/>
-      <c r="AA23" s="198"/>
-      <c r="AB23" s="198"/>
-      <c r="AC23" s="198"/>
-      <c r="AD23" s="198"/>
-      <c r="AE23" s="198"/>
-      <c r="AF23" s="198"/>
-      <c r="AG23" s="199"/>
+      <c r="Y23" s="194"/>
+      <c r="Z23" s="194"/>
+      <c r="AA23" s="194"/>
+      <c r="AB23" s="194"/>
+      <c r="AC23" s="194"/>
+      <c r="AD23" s="194"/>
+      <c r="AE23" s="194"/>
+      <c r="AF23" s="194"/>
+      <c r="AG23" s="195"/>
       <c r="AH23" s="131"/>
       <c r="AI23" s="132"/>
       <c r="AJ23" s="132"/>
@@ -56011,19 +56414,19 @@
       <c r="D24" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="193" t="s">
+      <c r="E24" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="193"/>
-      <c r="G24" s="193" t="s">
+      <c r="F24" s="196"/>
+      <c r="G24" s="196" t="s">
         <v>18</v>
       </c>
-      <c r="H24" s="193"/>
-      <c r="I24" s="193"/>
-      <c r="J24" s="193" t="s">
+      <c r="H24" s="196"/>
+      <c r="I24" s="196"/>
+      <c r="J24" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="K24" s="193"/>
+      <c r="K24" s="196"/>
       <c r="L24" s="135"/>
       <c r="M24" s="135"/>
       <c r="N24" s="135"/>
@@ -56045,19 +56448,19 @@
       <c r="Z24" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA24" s="193" t="s">
+      <c r="AA24" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AB24" s="193"/>
-      <c r="AC24" s="193" t="s">
+      <c r="AB24" s="196"/>
+      <c r="AC24" s="196" t="s">
         <v>18</v>
       </c>
-      <c r="AD24" s="193"/>
-      <c r="AE24" s="193"/>
-      <c r="AF24" s="193" t="s">
+      <c r="AD24" s="196"/>
+      <c r="AE24" s="196"/>
+      <c r="AF24" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="AG24" s="193"/>
+      <c r="AG24" s="196"/>
       <c r="AH24" s="136"/>
       <c r="AI24" s="133"/>
       <c r="AJ24" s="133"/>
@@ -56273,6 +56676,12 @@
         <f t="shared" ref="U28:U30" si="21">U27+5</f>
         <v>65</v>
       </c>
+      <c r="AD28" s="193" t="s">
+        <v>211</v>
+      </c>
+      <c r="AE28" s="194"/>
+      <c r="AF28" s="194"/>
+      <c r="AG28" s="195"/>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B29" s="152">
@@ -56317,6 +56726,10 @@
         <f t="shared" ref="U29:U31" si="22">U28+1</f>
         <v>66</v>
       </c>
+      <c r="AD29" s="205"/>
+      <c r="AE29" s="204"/>
+      <c r="AF29" s="204"/>
+      <c r="AG29" s="206"/>
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B30" s="152">
@@ -56361,6 +56774,10 @@
         <f t="shared" si="21"/>
         <v>71</v>
       </c>
+      <c r="AD30" s="205"/>
+      <c r="AE30" s="204"/>
+      <c r="AF30" s="204"/>
+      <c r="AG30" s="207"/>
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B31" s="152">
@@ -56405,6 +56822,10 @@
         <f t="shared" si="22"/>
         <v>72</v>
       </c>
+      <c r="AD31" s="205"/>
+      <c r="AE31" s="204"/>
+      <c r="AF31" s="204"/>
+      <c r="AG31" s="207"/>
     </row>
     <row r="32" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B32" s="152">
@@ -56442,6 +56863,10 @@
       <c r="N32" s="133">
         <v>96</v>
       </c>
+      <c r="AD32" s="208"/>
+      <c r="AE32" s="209"/>
+      <c r="AF32" s="209"/>
+      <c r="AG32" s="210"/>
     </row>
     <row r="33" spans="2:33" x14ac:dyDescent="0.25">
       <c r="C33" s="137"/>
@@ -56456,15 +56881,15 @@
       </c>
       <c r="Z34" s="202"/>
       <c r="AA34" s="202"/>
-      <c r="AB34" s="194" t="str">
+      <c r="AB34" s="197" t="str">
         <f>IF(AI25="1º Lugar","",AI25)</f>
         <v/>
       </c>
-      <c r="AC34" s="194"/>
-      <c r="AD34" s="194"/>
-      <c r="AE34" s="194"/>
-      <c r="AF34" s="194"/>
-      <c r="AG34" s="194"/>
+      <c r="AC34" s="197"/>
+      <c r="AD34" s="197"/>
+      <c r="AE34" s="197"/>
+      <c r="AF34" s="197"/>
+      <c r="AG34" s="197"/>
     </row>
     <row r="35" spans="2:33" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B35" s="140"/>
@@ -56476,15 +56901,15 @@
       </c>
       <c r="Z35" s="200"/>
       <c r="AA35" s="200"/>
-      <c r="AB35" s="195" t="str">
+      <c r="AB35" s="198" t="str">
         <f>IF(M57="2º Lugar","",M57)</f>
         <v/>
       </c>
-      <c r="AC35" s="195"/>
-      <c r="AD35" s="195"/>
-      <c r="AE35" s="195"/>
-      <c r="AF35" s="195"/>
-      <c r="AG35" s="195"/>
+      <c r="AC35" s="198"/>
+      <c r="AD35" s="198"/>
+      <c r="AE35" s="198"/>
+      <c r="AF35" s="198"/>
+      <c r="AG35" s="198"/>
     </row>
     <row r="36" spans="2:33" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B36" s="140"/>
@@ -56496,15 +56921,15 @@
       </c>
       <c r="Z36" s="201"/>
       <c r="AA36" s="201"/>
-      <c r="AB36" s="196" t="str">
+      <c r="AB36" s="199" t="str">
         <f>IF(AI19="3º Lugar","",AI19)</f>
         <v/>
       </c>
-      <c r="AC36" s="196"/>
-      <c r="AD36" s="196"/>
-      <c r="AE36" s="196"/>
-      <c r="AF36" s="196"/>
-      <c r="AG36" s="196"/>
+      <c r="AC36" s="199"/>
+      <c r="AD36" s="199"/>
+      <c r="AE36" s="199"/>
+      <c r="AF36" s="199"/>
+      <c r="AG36" s="199"/>
     </row>
     <row r="57" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C57" s="137"/>
@@ -56660,8 +57085,23 @@
       <c r="K82" s="45"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="e9SwIN3P1gzBH+IVoOp3qqE533HDYkDzheVXRVNRaqt2vhimaHXLKZ+8sDUopKeiKAT5et9NZBvuLRUJOa6zQg==" saltValue="pxuBsAAmB/Bn8sNidXdYpQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
-  <mergeCells count="30">
+  <sheetProtection algorithmName="SHA-512" hashValue="8JRv5B/B5jMSXJQTg3Gidv52YDGKsjKvo30SeOBaK6JSNYAMZQ/wPbZnASuXj0gcQnaFpGbQs8ZzG0RfUFK9kg==" saltValue="BbqaqtGKXaW/tQWh+QEg4w==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <mergeCells count="31">
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AB34:AG34"/>
+    <mergeCell ref="AB35:AG35"/>
+    <mergeCell ref="AB36:AG36"/>
+    <mergeCell ref="B23:K23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="Y35:AA35"/>
+    <mergeCell ref="Y36:AA36"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AE24"/>
+    <mergeCell ref="AF24:AG24"/>
+    <mergeCell ref="Y34:AA34"/>
+    <mergeCell ref="AD28:AG28"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:I4"/>
@@ -56678,158 +57118,144 @@
     <mergeCell ref="AF18:AG18"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="AC4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AB34:AG34"/>
-    <mergeCell ref="AB35:AG35"/>
-    <mergeCell ref="AB36:AG36"/>
-    <mergeCell ref="B23:K23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="Y35:AA35"/>
-    <mergeCell ref="Y36:AA36"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AE24"/>
-    <mergeCell ref="AF24:AG24"/>
-    <mergeCell ref="Y34:AA34"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A2 B2:K2 X9:AG10 X15:AG16 X20:AG21 B21:K22 AB34:AB36 A57:K58 H59:K61 B62:K71 B83:K1048576">
-    <cfRule type="cellIs" dxfId="27" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="76" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:B12 C4:K12">
-    <cfRule type="cellIs" dxfId="26" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="42" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13:K20">
-    <cfRule type="cellIs" dxfId="25" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="31" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B36 C24:K33">
-    <cfRule type="cellIs" dxfId="24" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="20" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F20">
-    <cfRule type="expression" dxfId="23" priority="30">
+    <cfRule type="expression" dxfId="43" priority="30">
       <formula>L5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F25:F32">
-    <cfRule type="expression" dxfId="22" priority="19">
+    <cfRule type="expression" dxfId="42" priority="19">
       <formula>L25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J20">
-    <cfRule type="expression" dxfId="21" priority="29">
+    <cfRule type="expression" dxfId="41" priority="29">
       <formula>L5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J25:J32">
-    <cfRule type="expression" dxfId="20" priority="18">
+    <cfRule type="expression" dxfId="40" priority="18">
       <formula>L25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K20">
-    <cfRule type="expression" dxfId="19" priority="21">
+    <cfRule type="expression" dxfId="39" priority="21">
       <formula>Q5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25:K32">
-    <cfRule type="expression" dxfId="18" priority="17">
+    <cfRule type="expression" dxfId="38" priority="17">
       <formula>Q25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W3:W24 A21:A34 I34:K34 Y34:AB34 Y34:Y36 A62:A1048576">
-    <cfRule type="cellIs" dxfId="17" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="77" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X3:X8 Y4:AG8">
-    <cfRule type="cellIs" dxfId="16" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="16" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X11:X14 Y12:AG14">
-    <cfRule type="cellIs" dxfId="15" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="12" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X17:X19 Y18:AG19">
-    <cfRule type="cellIs" dxfId="14" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="8" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X23:X25 Y24:AG25">
-    <cfRule type="cellIs" dxfId="13" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="4" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y34:AA36">
-    <cfRule type="expression" dxfId="12" priority="65">
+    <cfRule type="expression" dxfId="32" priority="65">
       <formula>AB34&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB5:AB8">
-    <cfRule type="expression" dxfId="11" priority="15">
+    <cfRule type="expression" dxfId="31" priority="15">
       <formula>AH5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB13:AB14">
-    <cfRule type="expression" dxfId="10" priority="11">
+    <cfRule type="expression" dxfId="30" priority="11">
       <formula>AH13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB19">
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="29" priority="7">
       <formula>AH19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB25">
-    <cfRule type="expression" dxfId="8" priority="3">
+    <cfRule type="expression" dxfId="28" priority="3">
       <formula>AH25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AF8">
-    <cfRule type="expression" dxfId="7" priority="14">
+    <cfRule type="expression" dxfId="27" priority="14">
       <formula>AH5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF13:AF14">
-    <cfRule type="expression" dxfId="6" priority="10">
+    <cfRule type="expression" dxfId="26" priority="10">
       <formula>AH13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF19">
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="25" priority="6">
       <formula>AH19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF25">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>AH25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG5:AG8">
-    <cfRule type="expression" dxfId="3" priority="13">
+    <cfRule type="expression" dxfId="23" priority="13">
       <formula>AM5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG13:AG14">
-    <cfRule type="expression" dxfId="2" priority="9">
+    <cfRule type="expression" dxfId="22" priority="9">
       <formula>AM13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG19">
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="21" priority="5">
       <formula>AM19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG25">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>AM25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -57454,6 +57880,12 @@
     <sortCondition ref="C59:C64"/>
   </sortState>
   <mergeCells count="16">
+    <mergeCell ref="N4:N6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="J4:J6"/>
+    <mergeCell ref="L4:L6"/>
     <mergeCell ref="AB4:AB6"/>
     <mergeCell ref="AD4:AD6"/>
     <mergeCell ref="AF4:AF6"/>
@@ -57464,12 +57896,6 @@
     <mergeCell ref="V4:V6"/>
     <mergeCell ref="X4:X6"/>
     <mergeCell ref="Z4:Z6"/>
-    <mergeCell ref="N4:N6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="J4:J6"/>
-    <mergeCell ref="L4:L6"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -57705,20 +58131,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -57741,6 +58167,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83E7837-68AD-48B2-A1AB-AAB452317AF5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="dc8c2798-6aba-4af7-93a4-b89253b03650"/>
@@ -57755,12 +58189,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Att Dia 4 Fase de 32
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9699A2C-6FD9-466F-82D7-B46D28F5B04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E09303-BA36-4D6D-A084-05BD5255E3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
@@ -2125,6 +2125,19 @@
     <xf numFmtId="0" fontId="39" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2135,6 +2148,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2161,15 +2183,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2194,142 +2207,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="91">
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2778,6 +2661,123 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -10007,31 +10007,31 @@
       <c r="I31" s="178" t="s">
         <v>206</v>
       </c>
-      <c r="J31" s="181" t="s">
+      <c r="J31" s="188" t="s">
         <v>81</v>
       </c>
-      <c r="K31" s="181"/>
-      <c r="L31" s="181"/>
+      <c r="K31" s="188"/>
+      <c r="L31" s="188"/>
     </row>
     <row r="32" spans="3:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="I32" s="179" t="s">
         <v>207</v>
       </c>
-      <c r="J32" s="182" t="s">
+      <c r="J32" s="189" t="s">
         <v>82</v>
       </c>
-      <c r="K32" s="182"/>
-      <c r="L32" s="182"/>
+      <c r="K32" s="189"/>
+      <c r="L32" s="189"/>
     </row>
     <row r="33" spans="9:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="I33" s="180" t="s">
         <v>208</v>
       </c>
-      <c r="J33" s="183" t="s">
+      <c r="J33" s="190" t="s">
         <v>83</v>
       </c>
-      <c r="K33" s="183"/>
-      <c r="L33" s="183"/>
+      <c r="K33" s="190"/>
+      <c r="L33" s="190"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="JhGV6VcDyvc3i9om8xFJD2TTjYS4KxdyrPHqfmvoUHY8jTzdLhnXdEDqhfq9o8QSGpM59e0FFua65Es5mRgoOA==" saltValue="uIq4f/wxSDvjcYmJtVUiRQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
@@ -11531,11 +11531,11 @@
       <c r="E3" s="91" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="184" t="s">
+      <c r="F3" s="191" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="184"/>
-      <c r="H3" s="184"/>
+      <c r="G3" s="191"/>
+      <c r="H3" s="191"/>
       <c r="I3" s="91" t="s">
         <v>17</v>
       </c>
@@ -15372,12 +15372,12 @@
         <f t="shared" ref="AR22:AR28" si="37">CODE(AQ22)</f>
         <v>70</v>
       </c>
-      <c r="BJ22" s="193" t="s">
+      <c r="BJ22" s="192" t="s">
         <v>211</v>
       </c>
-      <c r="BK22" s="194"/>
-      <c r="BL22" s="194"/>
-      <c r="BM22" s="195"/>
+      <c r="BK22" s="193"/>
+      <c r="BL22" s="193"/>
+      <c r="BM22" s="194"/>
     </row>
     <row r="23" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A23" s="45"/>
@@ -15511,10 +15511,10 @@
         <f t="shared" si="37"/>
         <v>69</v>
       </c>
-      <c r="BJ23" s="205"/>
-      <c r="BK23" s="204"/>
-      <c r="BL23" s="204"/>
-      <c r="BM23" s="206"/>
+      <c r="BJ23" s="182"/>
+      <c r="BK23" s="181"/>
+      <c r="BL23" s="181"/>
+      <c r="BM23" s="183"/>
     </row>
     <row r="24" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A24" s="45"/>
@@ -15671,10 +15671,10 @@
         <f t="shared" si="37"/>
         <v>76</v>
       </c>
-      <c r="BJ24" s="205"/>
-      <c r="BK24" s="204"/>
-      <c r="BL24" s="204"/>
-      <c r="BM24" s="207"/>
+      <c r="BJ24" s="182"/>
+      <c r="BK24" s="181"/>
+      <c r="BL24" s="181"/>
+      <c r="BM24" s="184"/>
     </row>
     <row r="25" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A25" s="45"/>
@@ -15831,10 +15831,10 @@
         <f t="shared" si="37"/>
         <v>66</v>
       </c>
-      <c r="BJ25" s="205"/>
-      <c r="BK25" s="204"/>
-      <c r="BL25" s="204"/>
-      <c r="BM25" s="207"/>
+      <c r="BJ25" s="182"/>
+      <c r="BK25" s="181"/>
+      <c r="BL25" s="181"/>
+      <c r="BM25" s="184"/>
     </row>
     <row r="26" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A26" s="45"/>
@@ -15991,10 +15991,10 @@
         <f t="shared" si="37"/>
         <v>74</v>
       </c>
-      <c r="BJ26" s="208"/>
-      <c r="BK26" s="209"/>
-      <c r="BL26" s="209"/>
-      <c r="BM26" s="210"/>
+      <c r="BJ26" s="185"/>
+      <c r="BK26" s="186"/>
+      <c r="BL26" s="186"/>
+      <c r="BM26" s="187"/>
     </row>
     <row r="27" spans="1:70" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="45"/>
@@ -22498,102 +22498,102 @@
     <mergeCell ref="BJ22:BM22"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A51 P3 B3:O51">
-    <cfRule type="cellIs" dxfId="19" priority="215" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="215" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A52:O75">
-    <cfRule type="cellIs" dxfId="18" priority="136" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="136" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:E9">
-    <cfRule type="cellIs" dxfId="17" priority="202" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="202" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:E21">
-    <cfRule type="cellIs" dxfId="16" priority="193" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="193" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:E33">
-    <cfRule type="cellIs" dxfId="15" priority="191" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="191" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C40:E45">
-    <cfRule type="cellIs" dxfId="14" priority="189" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="189" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C52:E57">
-    <cfRule type="cellIs" dxfId="13" priority="130" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="130" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C64:E69">
-    <cfRule type="cellIs" dxfId="12" priority="128" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="128" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:I9">
-    <cfRule type="cellIs" dxfId="11" priority="198" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="198" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16:I21">
-    <cfRule type="cellIs" dxfId="10" priority="188" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="188" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I28:I33">
-    <cfRule type="cellIs" dxfId="9" priority="187" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="187" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I40:I45">
-    <cfRule type="cellIs" dxfId="8" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="186" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I52:I57">
-    <cfRule type="cellIs" dxfId="7" priority="127" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="127" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I64:I69">
-    <cfRule type="cellIs" dxfId="6" priority="126" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="126" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:AN75">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6:AF7">
-    <cfRule type="expression" dxfId="4" priority="209">
+    <cfRule type="expression" dxfId="32" priority="209">
       <formula>AH6=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF12:AF13 AF18:AF19 AF24:AF25 AF30:AF31 AF36:AF37 AF42:AF43 AF48:AF49 AF54:AF55 AF60:AF61 AF66:AF67 AF72:AF73">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="31" priority="1">
       <formula>AH12=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AP5:BG17">
-    <cfRule type="cellIs" dxfId="2" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="83" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BI4:BR17">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="2" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BJ6:BJ13">
-    <cfRule type="expression" dxfId="0" priority="77">
+    <cfRule type="expression" dxfId="28" priority="77">
       <formula>BL6=3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22621,24 +22621,24 @@
   <sheetData>
     <row r="1" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B2" s="185" t="s">
+      <c r="B2" s="195" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="197" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="188"/>
-      <c r="E2" s="188"/>
-      <c r="F2" s="188"/>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="188"/>
-      <c r="J2" s="188"/>
-      <c r="K2" s="188"/>
-      <c r="L2" s="188"/>
-      <c r="M2" s="188"/>
-      <c r="N2" s="189"/>
-      <c r="O2" s="185"/>
+      <c r="D2" s="198"/>
+      <c r="E2" s="198"/>
+      <c r="F2" s="198"/>
+      <c r="G2" s="198"/>
+      <c r="H2" s="198"/>
+      <c r="I2" s="198"/>
+      <c r="J2" s="198"/>
+      <c r="K2" s="198"/>
+      <c r="L2" s="198"/>
+      <c r="M2" s="198"/>
+      <c r="N2" s="199"/>
+      <c r="O2" s="195"/>
       <c r="P2" s="5" t="s">
         <v>102</v>
       </c>
@@ -22665,22 +22665,22 @@
       </c>
     </row>
     <row r="3" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="186"/>
-      <c r="C3" s="190" t="s">
+      <c r="B3" s="196"/>
+      <c r="C3" s="200" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="191"/>
-      <c r="E3" s="191"/>
-      <c r="F3" s="191"/>
-      <c r="G3" s="191"/>
-      <c r="H3" s="191"/>
-      <c r="I3" s="191"/>
-      <c r="J3" s="191"/>
-      <c r="K3" s="191"/>
-      <c r="L3" s="191"/>
-      <c r="M3" s="191"/>
-      <c r="N3" s="192"/>
-      <c r="O3" s="186"/>
+      <c r="D3" s="201"/>
+      <c r="E3" s="201"/>
+      <c r="F3" s="201"/>
+      <c r="G3" s="201"/>
+      <c r="H3" s="201"/>
+      <c r="I3" s="201"/>
+      <c r="J3" s="201"/>
+      <c r="K3" s="201"/>
+      <c r="L3" s="201"/>
+      <c r="M3" s="201"/>
+      <c r="N3" s="202"/>
+      <c r="O3" s="196"/>
       <c r="P3" s="1" t="s">
         <v>103</v>
       </c>
@@ -54973,18 +54973,18 @@
     </row>
     <row r="3" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A3" s="130"/>
-      <c r="B3" s="193" t="s">
+      <c r="B3" s="192" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="194"/>
-      <c r="D3" s="194"/>
-      <c r="E3" s="194"/>
-      <c r="F3" s="194"/>
-      <c r="G3" s="194"/>
-      <c r="H3" s="194"/>
-      <c r="I3" s="194"/>
-      <c r="J3" s="194"/>
-      <c r="K3" s="195"/>
+      <c r="C3" s="193"/>
+      <c r="D3" s="193"/>
+      <c r="E3" s="193"/>
+      <c r="F3" s="193"/>
+      <c r="G3" s="193"/>
+      <c r="H3" s="193"/>
+      <c r="I3" s="193"/>
+      <c r="J3" s="193"/>
+      <c r="K3" s="194"/>
       <c r="L3" s="131"/>
       <c r="M3" s="132"/>
       <c r="N3" s="132"/>
@@ -54992,18 +54992,18 @@
       <c r="P3" s="132"/>
       <c r="Q3" s="132"/>
       <c r="W3" s="130"/>
-      <c r="X3" s="193" t="s">
+      <c r="X3" s="192" t="s">
         <v>73</v>
       </c>
-      <c r="Y3" s="194"/>
-      <c r="Z3" s="194"/>
-      <c r="AA3" s="194"/>
-      <c r="AB3" s="194"/>
-      <c r="AC3" s="194"/>
-      <c r="AD3" s="194"/>
-      <c r="AE3" s="194"/>
-      <c r="AF3" s="194"/>
-      <c r="AG3" s="195"/>
+      <c r="Y3" s="193"/>
+      <c r="Z3" s="193"/>
+      <c r="AA3" s="193"/>
+      <c r="AB3" s="193"/>
+      <c r="AC3" s="193"/>
+      <c r="AD3" s="193"/>
+      <c r="AE3" s="193"/>
+      <c r="AF3" s="193"/>
+      <c r="AG3" s="194"/>
       <c r="AH3" s="131"/>
       <c r="AI3" s="132"/>
       <c r="AJ3" s="132"/>
@@ -55020,19 +55020,19 @@
       <c r="D4" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="196" t="s">
+      <c r="E4" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="196"/>
-      <c r="G4" s="196" t="s">
+      <c r="F4" s="203"/>
+      <c r="G4" s="203" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="196"/>
-      <c r="I4" s="196"/>
-      <c r="J4" s="196" t="s">
+      <c r="H4" s="203"/>
+      <c r="I4" s="203"/>
+      <c r="J4" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="196"/>
+      <c r="K4" s="203"/>
       <c r="L4" s="135"/>
       <c r="M4" s="135"/>
       <c r="N4" s="135"/>
@@ -55047,19 +55047,19 @@
       <c r="Z4" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="196" t="s">
+      <c r="AA4" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AB4" s="196"/>
-      <c r="AC4" s="196" t="s">
+      <c r="AB4" s="203"/>
+      <c r="AC4" s="203" t="s">
         <v>18</v>
       </c>
-      <c r="AD4" s="196"/>
-      <c r="AE4" s="196"/>
-      <c r="AF4" s="196" t="s">
+      <c r="AD4" s="203"/>
+      <c r="AE4" s="203"/>
+      <c r="AF4" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AG4" s="196"/>
+      <c r="AG4" s="203"/>
       <c r="AH4" s="136"/>
       <c r="AI4" s="133"/>
       <c r="AJ4" s="133"/>
@@ -55619,18 +55619,18 @@
         <v>12</v>
       </c>
       <c r="W11" s="130"/>
-      <c r="X11" s="193" t="s">
+      <c r="X11" s="192" t="s">
         <v>74</v>
       </c>
-      <c r="Y11" s="194"/>
-      <c r="Z11" s="194"/>
-      <c r="AA11" s="194"/>
-      <c r="AB11" s="194"/>
-      <c r="AC11" s="194"/>
-      <c r="AD11" s="194"/>
-      <c r="AE11" s="194"/>
-      <c r="AF11" s="194"/>
-      <c r="AG11" s="195"/>
+      <c r="Y11" s="193"/>
+      <c r="Z11" s="193"/>
+      <c r="AA11" s="193"/>
+      <c r="AB11" s="193"/>
+      <c r="AC11" s="193"/>
+      <c r="AD11" s="193"/>
+      <c r="AE11" s="193"/>
+      <c r="AF11" s="193"/>
+      <c r="AG11" s="194"/>
       <c r="AH11" s="131"/>
       <c r="AI11" s="132"/>
       <c r="AJ11" s="132"/>
@@ -55653,11 +55653,15 @@
         <v>Inglaterra</v>
       </c>
       <c r="F12" s="149"/>
-      <c r="G12" s="123"/>
+      <c r="G12" s="123">
+        <v>2</v>
+      </c>
       <c r="H12" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="123"/>
+      <c r="I12" s="123">
+        <v>1</v>
+      </c>
       <c r="J12" s="150"/>
       <c r="K12" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R15,"3º E, H, I, J ou K")</f>
@@ -55669,7 +55673,7 @@
       </c>
       <c r="M12" s="133" t="str">
         <f>IF(OR(G12="",I12=""),"Vencedor 80",IF(G12&lt;&gt;I12,IF(G12&gt;I12,E12,K12),IF(SUM(F12:G12)=SUM(I12:J12),"Vencedor 80",IF(SUM(F12:G12)&gt;SUM(I12:J12),E12,K12))))</f>
-        <v>Vencedor 80</v>
+        <v>Inglaterra</v>
       </c>
       <c r="N12" s="133">
         <v>80</v>
@@ -55700,19 +55704,19 @@
       <c r="Z12" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA12" s="196" t="s">
+      <c r="AA12" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AB12" s="196"/>
-      <c r="AC12" s="196" t="s">
+      <c r="AB12" s="203"/>
+      <c r="AC12" s="203" t="s">
         <v>18</v>
       </c>
-      <c r="AD12" s="196"/>
-      <c r="AE12" s="196"/>
-      <c r="AF12" s="196" t="s">
+      <c r="AD12" s="203"/>
+      <c r="AE12" s="203"/>
+      <c r="AF12" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AG12" s="196"/>
+      <c r="AG12" s="203"/>
       <c r="AH12" s="136"/>
       <c r="AI12" s="133"/>
       <c r="AJ12" s="133"/>
@@ -55735,11 +55739,15 @@
         <v>Estados Unidos</v>
       </c>
       <c r="F13" s="149"/>
-      <c r="G13" s="123"/>
+      <c r="G13" s="123">
+        <v>2</v>
+      </c>
       <c r="H13" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="123"/>
+      <c r="I13" s="123">
+        <v>0</v>
+      </c>
       <c r="J13" s="150"/>
       <c r="K13" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R10,"3º B, E, F, I ou J")</f>
@@ -55751,7 +55759,7 @@
       </c>
       <c r="M13" s="133" t="str">
         <f>IF(OR(G13="",I13=""),"Vencedor 81",IF(G13&lt;&gt;I13,IF(G13&gt;I13,E13,K13),IF(SUM(F13:G13)=SUM(I13:J13),"Vencedor 81",IF(SUM(F13:G13)&gt;SUM(I13:J13),E13,K13))))</f>
-        <v>Vencedor 81</v>
+        <v>Estados Unidos</v>
       </c>
       <c r="N13" s="133">
         <v>81</v>
@@ -55827,11 +55835,15 @@
         <v>Bélgica</v>
       </c>
       <c r="F14" s="149"/>
-      <c r="G14" s="123"/>
+      <c r="G14" s="123">
+        <v>3</v>
+      </c>
       <c r="H14" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I14" s="123"/>
+      <c r="I14" s="123">
+        <v>2</v>
+      </c>
       <c r="J14" s="150"/>
       <c r="K14" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R12,"3º A, E, H, I ou J")</f>
@@ -55843,7 +55855,7 @@
       </c>
       <c r="M14" s="133" t="str">
         <f>IF(OR(G14="",I14=""),"Vencedor 82",IF(G14&lt;&gt;I14,IF(G14&gt;I14,E14,K14),IF(SUM(F14:G14)=SUM(I14:J14),"Vencedor 82",IF(SUM(F14:G14)&gt;SUM(I14:J14),E14,K14))))</f>
-        <v>Vencedor 82</v>
+        <v>Bélgica</v>
       </c>
       <c r="N14" s="133">
         <v>82</v>
@@ -56087,18 +56099,18 @@
         <v>30</v>
       </c>
       <c r="W17" s="130"/>
-      <c r="X17" s="193" t="s">
+      <c r="X17" s="192" t="s">
         <v>77</v>
       </c>
-      <c r="Y17" s="194"/>
-      <c r="Z17" s="194"/>
-      <c r="AA17" s="194"/>
-      <c r="AB17" s="194"/>
-      <c r="AC17" s="194"/>
-      <c r="AD17" s="194"/>
-      <c r="AE17" s="194"/>
-      <c r="AF17" s="194"/>
-      <c r="AG17" s="195"/>
+      <c r="Y17" s="193"/>
+      <c r="Z17" s="193"/>
+      <c r="AA17" s="193"/>
+      <c r="AB17" s="193"/>
+      <c r="AC17" s="193"/>
+      <c r="AD17" s="193"/>
+      <c r="AE17" s="193"/>
+      <c r="AF17" s="193"/>
+      <c r="AG17" s="194"/>
       <c r="AH17" s="131"/>
       <c r="AI17" s="132"/>
       <c r="AJ17" s="132"/>
@@ -56157,19 +56169,19 @@
       <c r="Z18" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA18" s="196" t="s">
+      <c r="AA18" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AB18" s="196"/>
-      <c r="AC18" s="196" t="s">
+      <c r="AB18" s="203"/>
+      <c r="AC18" s="203" t="s">
         <v>18</v>
       </c>
-      <c r="AD18" s="196"/>
-      <c r="AE18" s="196"/>
-      <c r="AF18" s="196" t="s">
+      <c r="AD18" s="203"/>
+      <c r="AE18" s="203"/>
+      <c r="AF18" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AG18" s="196"/>
+      <c r="AG18" s="203"/>
       <c r="AH18" s="136"/>
       <c r="AI18" s="133"/>
       <c r="AJ18" s="133"/>
@@ -56361,18 +56373,18 @@
     </row>
     <row r="23" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A23" s="130"/>
-      <c r="B23" s="193" t="s">
+      <c r="B23" s="192" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="194"/>
-      <c r="D23" s="194"/>
-      <c r="E23" s="194"/>
-      <c r="F23" s="194"/>
-      <c r="G23" s="194"/>
-      <c r="H23" s="194"/>
-      <c r="I23" s="194"/>
-      <c r="J23" s="194"/>
-      <c r="K23" s="195"/>
+      <c r="C23" s="193"/>
+      <c r="D23" s="193"/>
+      <c r="E23" s="193"/>
+      <c r="F23" s="193"/>
+      <c r="G23" s="193"/>
+      <c r="H23" s="193"/>
+      <c r="I23" s="193"/>
+      <c r="J23" s="193"/>
+      <c r="K23" s="194"/>
       <c r="L23" s="131"/>
       <c r="M23" s="132"/>
       <c r="N23" s="132"/>
@@ -56387,18 +56399,18 @@
         <v>48</v>
       </c>
       <c r="W23" s="45"/>
-      <c r="X23" s="193" t="s">
+      <c r="X23" s="192" t="s">
         <v>79</v>
       </c>
-      <c r="Y23" s="194"/>
-      <c r="Z23" s="194"/>
-      <c r="AA23" s="194"/>
-      <c r="AB23" s="194"/>
-      <c r="AC23" s="194"/>
-      <c r="AD23" s="194"/>
-      <c r="AE23" s="194"/>
-      <c r="AF23" s="194"/>
-      <c r="AG23" s="195"/>
+      <c r="Y23" s="193"/>
+      <c r="Z23" s="193"/>
+      <c r="AA23" s="193"/>
+      <c r="AB23" s="193"/>
+      <c r="AC23" s="193"/>
+      <c r="AD23" s="193"/>
+      <c r="AE23" s="193"/>
+      <c r="AF23" s="193"/>
+      <c r="AG23" s="194"/>
       <c r="AH23" s="131"/>
       <c r="AI23" s="132"/>
       <c r="AJ23" s="132"/>
@@ -56414,19 +56426,19 @@
       <c r="D24" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="196" t="s">
+      <c r="E24" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="196"/>
-      <c r="G24" s="196" t="s">
+      <c r="F24" s="203"/>
+      <c r="G24" s="203" t="s">
         <v>18</v>
       </c>
-      <c r="H24" s="196"/>
-      <c r="I24" s="196"/>
-      <c r="J24" s="196" t="s">
+      <c r="H24" s="203"/>
+      <c r="I24" s="203"/>
+      <c r="J24" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="K24" s="196"/>
+      <c r="K24" s="203"/>
       <c r="L24" s="135"/>
       <c r="M24" s="135"/>
       <c r="N24" s="135"/>
@@ -56448,19 +56460,19 @@
       <c r="Z24" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AA24" s="196" t="s">
+      <c r="AA24" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AB24" s="196"/>
-      <c r="AC24" s="196" t="s">
+      <c r="AB24" s="203"/>
+      <c r="AC24" s="203" t="s">
         <v>18</v>
       </c>
-      <c r="AD24" s="196"/>
-      <c r="AE24" s="196"/>
-      <c r="AF24" s="196" t="s">
+      <c r="AD24" s="203"/>
+      <c r="AE24" s="203"/>
+      <c r="AF24" s="203" t="s">
         <v>17</v>
       </c>
-      <c r="AG24" s="196"/>
+      <c r="AG24" s="203"/>
       <c r="AH24" s="136"/>
       <c r="AI24" s="133"/>
       <c r="AJ24" s="133"/>
@@ -56656,7 +56668,7 @@
       <c r="J28" s="150"/>
       <c r="K28" s="151" t="str">
         <f>M12</f>
-        <v>Vencedor 80</v>
+        <v>Inglaterra</v>
       </c>
       <c r="L28" s="136" t="str">
         <f t="shared" si="18"/>
@@ -56676,12 +56688,12 @@
         <f t="shared" ref="U28:U30" si="21">U27+5</f>
         <v>65</v>
       </c>
-      <c r="AD28" s="193" t="s">
+      <c r="AD28" s="192" t="s">
         <v>211</v>
       </c>
-      <c r="AE28" s="194"/>
-      <c r="AF28" s="194"/>
-      <c r="AG28" s="195"/>
+      <c r="AE28" s="193"/>
+      <c r="AF28" s="193"/>
+      <c r="AG28" s="194"/>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B29" s="152">
@@ -56726,10 +56738,10 @@
         <f t="shared" ref="U29:U31" si="22">U28+1</f>
         <v>66</v>
       </c>
-      <c r="AD29" s="205"/>
-      <c r="AE29" s="204"/>
-      <c r="AF29" s="204"/>
-      <c r="AG29" s="206"/>
+      <c r="AD29" s="182"/>
+      <c r="AE29" s="181"/>
+      <c r="AF29" s="181"/>
+      <c r="AG29" s="183"/>
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B30" s="152">
@@ -56743,7 +56755,7 @@
       </c>
       <c r="E30" s="106" t="str">
         <f>M13</f>
-        <v>Vencedor 81</v>
+        <v>Estados Unidos</v>
       </c>
       <c r="F30" s="149"/>
       <c r="G30" s="123"/>
@@ -56754,7 +56766,7 @@
       <c r="J30" s="150"/>
       <c r="K30" s="151" t="str">
         <f>M14</f>
-        <v>Vencedor 82</v>
+        <v>Bélgica</v>
       </c>
       <c r="L30" s="136" t="str">
         <f t="shared" si="18"/>
@@ -56774,10 +56786,10 @@
         <f t="shared" si="21"/>
         <v>71</v>
       </c>
-      <c r="AD30" s="205"/>
-      <c r="AE30" s="204"/>
-      <c r="AF30" s="204"/>
-      <c r="AG30" s="207"/>
+      <c r="AD30" s="182"/>
+      <c r="AE30" s="181"/>
+      <c r="AF30" s="181"/>
+      <c r="AG30" s="184"/>
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B31" s="152">
@@ -56822,10 +56834,10 @@
         <f t="shared" si="22"/>
         <v>72</v>
       </c>
-      <c r="AD31" s="205"/>
-      <c r="AE31" s="204"/>
-      <c r="AF31" s="204"/>
-      <c r="AG31" s="207"/>
+      <c r="AD31" s="182"/>
+      <c r="AE31" s="181"/>
+      <c r="AF31" s="181"/>
+      <c r="AG31" s="184"/>
     </row>
     <row r="32" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B32" s="152">
@@ -56863,10 +56875,10 @@
       <c r="N32" s="133">
         <v>96</v>
       </c>
-      <c r="AD32" s="208"/>
-      <c r="AE32" s="209"/>
-      <c r="AF32" s="209"/>
-      <c r="AG32" s="210"/>
+      <c r="AD32" s="185"/>
+      <c r="AE32" s="186"/>
+      <c r="AF32" s="186"/>
+      <c r="AG32" s="187"/>
     </row>
     <row r="33" spans="2:33" x14ac:dyDescent="0.25">
       <c r="C33" s="137"/>
@@ -56876,60 +56888,60 @@
       <c r="X34" s="158" t="s">
         <v>206</v>
       </c>
-      <c r="Y34" s="202" t="s">
+      <c r="Y34" s="209" t="s">
         <v>81</v>
       </c>
-      <c r="Z34" s="202"/>
-      <c r="AA34" s="202"/>
-      <c r="AB34" s="197" t="str">
+      <c r="Z34" s="209"/>
+      <c r="AA34" s="209"/>
+      <c r="AB34" s="204" t="str">
         <f>IF(AI25="1º Lugar","",AI25)</f>
         <v/>
       </c>
-      <c r="AC34" s="197"/>
-      <c r="AD34" s="197"/>
-      <c r="AE34" s="197"/>
-      <c r="AF34" s="197"/>
-      <c r="AG34" s="197"/>
+      <c r="AC34" s="204"/>
+      <c r="AD34" s="204"/>
+      <c r="AE34" s="204"/>
+      <c r="AF34" s="204"/>
+      <c r="AG34" s="204"/>
     </row>
     <row r="35" spans="2:33" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B35" s="140"/>
       <c r="X35" s="159" t="s">
         <v>207</v>
       </c>
-      <c r="Y35" s="200" t="s">
+      <c r="Y35" s="207" t="s">
         <v>82</v>
       </c>
-      <c r="Z35" s="200"/>
-      <c r="AA35" s="200"/>
-      <c r="AB35" s="198" t="str">
+      <c r="Z35" s="207"/>
+      <c r="AA35" s="207"/>
+      <c r="AB35" s="205" t="str">
         <f>IF(M57="2º Lugar","",M57)</f>
         <v/>
       </c>
-      <c r="AC35" s="198"/>
-      <c r="AD35" s="198"/>
-      <c r="AE35" s="198"/>
-      <c r="AF35" s="198"/>
-      <c r="AG35" s="198"/>
+      <c r="AC35" s="205"/>
+      <c r="AD35" s="205"/>
+      <c r="AE35" s="205"/>
+      <c r="AF35" s="205"/>
+      <c r="AG35" s="205"/>
     </row>
     <row r="36" spans="2:33" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B36" s="140"/>
       <c r="X36" s="160" t="s">
         <v>208</v>
       </c>
-      <c r="Y36" s="201" t="s">
+      <c r="Y36" s="208" t="s">
         <v>83</v>
       </c>
-      <c r="Z36" s="201"/>
-      <c r="AA36" s="201"/>
-      <c r="AB36" s="199" t="str">
+      <c r="Z36" s="208"/>
+      <c r="AA36" s="208"/>
+      <c r="AB36" s="206" t="str">
         <f>IF(AI19="3º Lugar","",AI19)</f>
         <v/>
       </c>
-      <c r="AC36" s="199"/>
-      <c r="AD36" s="199"/>
-      <c r="AE36" s="199"/>
-      <c r="AF36" s="199"/>
-      <c r="AG36" s="199"/>
+      <c r="AC36" s="206"/>
+      <c r="AD36" s="206"/>
+      <c r="AE36" s="206"/>
+      <c r="AF36" s="206"/>
+      <c r="AG36" s="206"/>
     </row>
     <row r="57" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C57" s="137"/>
@@ -57120,142 +57132,142 @@
     <mergeCell ref="AC4:AE4"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A2 B2:K2 X9:AG10 X15:AG16 X20:AG21 B21:K22 AB34:AB36 A57:K58 H59:K61 B62:K71 B83:K1048576">
-    <cfRule type="cellIs" dxfId="47" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="76" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:B12 C4:K12">
-    <cfRule type="cellIs" dxfId="46" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="42" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13:K20">
-    <cfRule type="cellIs" dxfId="45" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="31" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B36 C24:K33">
-    <cfRule type="cellIs" dxfId="44" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="20" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F20">
-    <cfRule type="expression" dxfId="43" priority="30">
+    <cfRule type="expression" dxfId="23" priority="30">
       <formula>L5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F25:F32">
-    <cfRule type="expression" dxfId="42" priority="19">
+    <cfRule type="expression" dxfId="22" priority="19">
       <formula>L25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J20">
-    <cfRule type="expression" dxfId="41" priority="29">
+    <cfRule type="expression" dxfId="21" priority="29">
       <formula>L5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J25:J32">
-    <cfRule type="expression" dxfId="40" priority="18">
+    <cfRule type="expression" dxfId="20" priority="18">
       <formula>L25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K20">
-    <cfRule type="expression" dxfId="39" priority="21">
+    <cfRule type="expression" dxfId="19" priority="21">
       <formula>Q5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25:K32">
-    <cfRule type="expression" dxfId="38" priority="17">
+    <cfRule type="expression" dxfId="18" priority="17">
       <formula>Q25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W3:W24 A21:A34 I34:K34 Y34:AB34 Y34:Y36 A62:A1048576">
-    <cfRule type="cellIs" dxfId="37" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="77" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X3:X8 Y4:AG8">
-    <cfRule type="cellIs" dxfId="36" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="16" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X11:X14 Y12:AG14">
-    <cfRule type="cellIs" dxfId="35" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="12" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X17:X19 Y18:AG19">
-    <cfRule type="cellIs" dxfId="34" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="8" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X23:X25 Y24:AG25">
-    <cfRule type="cellIs" dxfId="33" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="4" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y34:AA36">
-    <cfRule type="expression" dxfId="32" priority="65">
+    <cfRule type="expression" dxfId="12" priority="65">
       <formula>AB34&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB5:AB8">
-    <cfRule type="expression" dxfId="31" priority="15">
+    <cfRule type="expression" dxfId="11" priority="15">
       <formula>AH5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB13:AB14">
-    <cfRule type="expression" dxfId="30" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>AH13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB19">
-    <cfRule type="expression" dxfId="29" priority="7">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AH19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB25">
-    <cfRule type="expression" dxfId="28" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>AH25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AF8">
-    <cfRule type="expression" dxfId="27" priority="14">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>AH5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF13:AF14">
-    <cfRule type="expression" dxfId="26" priority="10">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>AH13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF19">
-    <cfRule type="expression" dxfId="25" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>AH19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF25">
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>AH25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG5:AG8">
-    <cfRule type="expression" dxfId="23" priority="13">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>AM5="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG13:AG14">
-    <cfRule type="expression" dxfId="22" priority="9">
+    <cfRule type="expression" dxfId="2" priority="9">
       <formula>AM13="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG19">
-    <cfRule type="expression" dxfId="21" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>AM19="emp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG25">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>AM25="emp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -57322,64 +57334,64 @@
       <c r="C4" s="169" t="s">
         <v>161</v>
       </c>
-      <c r="D4" s="203"/>
-      <c r="F4" s="203"/>
-      <c r="H4" s="203"/>
-      <c r="J4" s="203"/>
-      <c r="L4" s="203"/>
-      <c r="N4" s="203"/>
-      <c r="P4" s="203"/>
-      <c r="R4" s="203"/>
-      <c r="T4" s="203"/>
-      <c r="V4" s="203"/>
-      <c r="X4" s="203"/>
-      <c r="Z4" s="203"/>
-      <c r="AB4" s="203"/>
-      <c r="AD4" s="203"/>
-      <c r="AF4" s="203"/>
-      <c r="AH4" s="203"/>
+      <c r="D4" s="210"/>
+      <c r="F4" s="210"/>
+      <c r="H4" s="210"/>
+      <c r="J4" s="210"/>
+      <c r="L4" s="210"/>
+      <c r="N4" s="210"/>
+      <c r="P4" s="210"/>
+      <c r="R4" s="210"/>
+      <c r="T4" s="210"/>
+      <c r="V4" s="210"/>
+      <c r="X4" s="210"/>
+      <c r="Z4" s="210"/>
+      <c r="AB4" s="210"/>
+      <c r="AD4" s="210"/>
+      <c r="AF4" s="210"/>
+      <c r="AH4" s="210"/>
     </row>
     <row r="5" spans="2:34" x14ac:dyDescent="0.3">
       <c r="C5" s="169" t="s">
         <v>163</v>
       </c>
-      <c r="D5" s="203"/>
-      <c r="F5" s="203"/>
-      <c r="H5" s="203"/>
-      <c r="J5" s="203"/>
-      <c r="L5" s="203"/>
-      <c r="N5" s="203"/>
-      <c r="P5" s="203"/>
-      <c r="R5" s="203"/>
-      <c r="T5" s="203"/>
-      <c r="V5" s="203"/>
-      <c r="X5" s="203"/>
-      <c r="Z5" s="203"/>
-      <c r="AB5" s="203"/>
-      <c r="AD5" s="203"/>
-      <c r="AF5" s="203"/>
-      <c r="AH5" s="203"/>
+      <c r="D5" s="210"/>
+      <c r="F5" s="210"/>
+      <c r="H5" s="210"/>
+      <c r="J5" s="210"/>
+      <c r="L5" s="210"/>
+      <c r="N5" s="210"/>
+      <c r="P5" s="210"/>
+      <c r="R5" s="210"/>
+      <c r="T5" s="210"/>
+      <c r="V5" s="210"/>
+      <c r="X5" s="210"/>
+      <c r="Z5" s="210"/>
+      <c r="AB5" s="210"/>
+      <c r="AD5" s="210"/>
+      <c r="AF5" s="210"/>
+      <c r="AH5" s="210"/>
     </row>
     <row r="6" spans="2:34" x14ac:dyDescent="0.3">
       <c r="C6" s="169" t="s">
         <v>162</v>
       </c>
-      <c r="D6" s="203"/>
-      <c r="F6" s="203"/>
-      <c r="H6" s="203"/>
-      <c r="J6" s="203"/>
-      <c r="L6" s="203"/>
-      <c r="N6" s="203"/>
-      <c r="P6" s="203"/>
-      <c r="R6" s="203"/>
-      <c r="T6" s="203"/>
-      <c r="V6" s="203"/>
-      <c r="X6" s="203"/>
-      <c r="Z6" s="203"/>
-      <c r="AB6" s="203"/>
-      <c r="AD6" s="203"/>
-      <c r="AF6" s="203"/>
-      <c r="AH6" s="203"/>
+      <c r="D6" s="210"/>
+      <c r="F6" s="210"/>
+      <c r="H6" s="210"/>
+      <c r="J6" s="210"/>
+      <c r="L6" s="210"/>
+      <c r="N6" s="210"/>
+      <c r="P6" s="210"/>
+      <c r="R6" s="210"/>
+      <c r="T6" s="210"/>
+      <c r="V6" s="210"/>
+      <c r="X6" s="210"/>
+      <c r="Z6" s="210"/>
+      <c r="AB6" s="210"/>
+      <c r="AD6" s="210"/>
+      <c r="AF6" s="210"/>
+      <c r="AH6" s="210"/>
     </row>
     <row r="7" spans="2:34" x14ac:dyDescent="0.3">
       <c r="C7" s="169" t="s">

</xml_diff>

<commit_message>
Att Oitavas dia 2
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E09303-BA36-4D6D-A084-05BD5255E3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED78202-39B0-4377-A87D-8EDFD748F56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
@@ -55119,7 +55119,7 @@
       </c>
       <c r="AA5" s="106" t="str">
         <f>M25</f>
-        <v>Vencedor 89</v>
+        <v>França</v>
       </c>
       <c r="AB5" s="149"/>
       <c r="AC5" s="123"/>
@@ -55130,7 +55130,7 @@
       <c r="AF5" s="150"/>
       <c r="AG5" s="151" t="str">
         <f>M26</f>
-        <v>Vencedor 90</v>
+        <v>Marrocos</v>
       </c>
       <c r="AH5" s="136" t="str">
         <f>IF(OR(AC5="",AE5=""),"",IF(AC5=AE5,"emp",""))</f>
@@ -55287,7 +55287,7 @@
       </c>
       <c r="AA7" s="106" t="str">
         <f>M27</f>
-        <v>Vencedor 91</v>
+        <v>Noruega</v>
       </c>
       <c r="AB7" s="149"/>
       <c r="AC7" s="123"/>
@@ -55298,7 +55298,7 @@
       <c r="AF7" s="150"/>
       <c r="AG7" s="151" t="str">
         <f>M28</f>
-        <v>Vencedor 92</v>
+        <v>Inglaterra</v>
       </c>
       <c r="AH7" s="136" t="str">
         <f t="shared" si="1"/>
@@ -55883,7 +55883,7 @@
         <v>76</v>
       </c>
       <c r="Y14" s="148">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="Z14" s="36" t="s">
         <v>46</v>
@@ -55931,11 +55931,15 @@
         <v>Portugal</v>
       </c>
       <c r="F15" s="149"/>
-      <c r="G15" s="123"/>
+      <c r="G15" s="123">
+        <v>2</v>
+      </c>
       <c r="H15" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I15" s="123"/>
+      <c r="I15" s="123">
+        <v>1</v>
+      </c>
       <c r="J15" s="150"/>
       <c r="K15" s="151" t="str">
         <f>IF('Fase de Grupos'!AH73=3,'Fase de Grupos'!AF73,"2º do Grupo L")</f>
@@ -55947,7 +55951,7 @@
       </c>
       <c r="M15" s="133" t="str">
         <f>IF(OR(G15="",I15=""),"Vencedor 83",IF(G15&lt;&gt;I15,IF(G15&gt;I15,E15,K15),IF(SUM(F15:G15)=SUM(I15:J15),"Vencedor 83",IF(SUM(F15:G15)&gt;SUM(I15:J15),E15,K15))))</f>
-        <v>Vencedor 83</v>
+        <v>Portugal</v>
       </c>
       <c r="N15" s="133">
         <v>83</v>
@@ -56006,11 +56010,15 @@
         <v>Espanha</v>
       </c>
       <c r="F16" s="149"/>
-      <c r="G16" s="123"/>
+      <c r="G16" s="123">
+        <v>3</v>
+      </c>
       <c r="H16" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I16" s="123"/>
+      <c r="I16" s="123">
+        <v>0</v>
+      </c>
       <c r="J16" s="150"/>
       <c r="K16" s="151" t="str">
         <f>IF('Fase de Grupos'!AH61=3,'Fase de Grupos'!AF61,"2º do Grupo J")</f>
@@ -56022,7 +56030,7 @@
       </c>
       <c r="M16" s="133" t="str">
         <f>IF(OR(G16="",I16=""),"Vencedor 84",IF(G16&lt;&gt;I16,IF(G16&gt;I16,E16,K16),IF(SUM(F16:G16)=SUM(I16:J16),"Vencedor 84",IF(SUM(F16:G16)&gt;SUM(I16:J16),E16,K16))))</f>
-        <v>Vencedor 84</v>
+        <v>Espanha</v>
       </c>
       <c r="N16" s="133">
         <v>84</v>
@@ -56070,11 +56078,15 @@
         <v>Suiça</v>
       </c>
       <c r="F17" s="149"/>
-      <c r="G17" s="123"/>
+      <c r="G17" s="123">
+        <v>2</v>
+      </c>
       <c r="H17" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I17" s="123"/>
+      <c r="I17" s="123">
+        <v>0</v>
+      </c>
       <c r="J17" s="150"/>
       <c r="K17" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R9,"3º E, F, G, I ou J")</f>
@@ -56086,7 +56098,7 @@
       </c>
       <c r="M17" s="133" t="str">
         <f>IF(OR(G17="",I17=""),"Vencedor 85",IF(G17&lt;&gt;I17,IF(G17&gt;I17,E17,K17),IF(SUM(F17:G17)=SUM(I17:J17),"Vencedor 85",IF(SUM(F17:G17)&gt;SUM(I17:J17),E17,K17))))</f>
-        <v>Vencedor 85</v>
+        <v>Suiça</v>
       </c>
       <c r="N17" s="133">
         <v>85</v>
@@ -56133,11 +56145,15 @@
         <v>Argentina</v>
       </c>
       <c r="F18" s="149"/>
-      <c r="G18" s="123"/>
+      <c r="G18" s="123">
+        <v>3</v>
+      </c>
       <c r="H18" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="123"/>
+      <c r="I18" s="123">
+        <v>2</v>
+      </c>
       <c r="J18" s="150"/>
       <c r="K18" s="151" t="str">
         <f>IF('Fase de Grupos'!AH49=3,'Fase de Grupos'!AF49,"2º do Grupo H")</f>
@@ -56149,7 +56165,7 @@
       </c>
       <c r="M18" s="133" t="str">
         <f>IF(OR(G18="",I18=""),"Vencedor 86",IF(G18&lt;&gt;I18,IF(G18&gt;I18,E18,K18),IF(SUM(F18:G18)=SUM(I18:J18),"Vencedor 86",IF(SUM(F18:G18)&gt;SUM(I18:J18),E18,K18))))</f>
-        <v>Vencedor 86</v>
+        <v>Argentina</v>
       </c>
       <c r="N18" s="133">
         <v>86</v>
@@ -56204,11 +56220,15 @@
         <v>Colômbia</v>
       </c>
       <c r="F19" s="149"/>
-      <c r="G19" s="123"/>
+      <c r="G19" s="123">
+        <v>1</v>
+      </c>
       <c r="H19" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I19" s="123"/>
+      <c r="I19" s="123">
+        <v>1</v>
+      </c>
       <c r="J19" s="150"/>
       <c r="K19" s="151" t="str">
         <f>IF('Fase de Grupos'!$BL$18=36,R14,"3º D, E, I, J ou L")</f>
@@ -56216,7 +56236,7 @@
       </c>
       <c r="L19" s="136" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>emp</v>
       </c>
       <c r="M19" s="133" t="str">
         <f>IF(OR(G19="",I19=""),"Vencedor 87",IF(G19&lt;&gt;I19,IF(G19&gt;I19,E19,K19),IF(SUM(F19:G19)=SUM(I19:J19),"Vencedor 87",IF(SUM(F19:G19)&gt;SUM(I19:J19),E19,K19))))</f>
@@ -56284,24 +56304,32 @@
         <f>IF('Fase de Grupos'!AH25=3,'Fase de Grupos'!AF25,"2º do Grupo D")</f>
         <v>Austrália</v>
       </c>
-      <c r="F20" s="149"/>
-      <c r="G20" s="123"/>
+      <c r="F20" s="149">
+        <v>2</v>
+      </c>
+      <c r="G20" s="123">
+        <v>1</v>
+      </c>
       <c r="H20" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I20" s="123"/>
-      <c r="J20" s="150"/>
+      <c r="I20" s="123">
+        <v>1</v>
+      </c>
+      <c r="J20" s="150">
+        <v>4</v>
+      </c>
       <c r="K20" s="151" t="str">
         <f>IF('Fase de Grupos'!AH43=3,'Fase de Grupos'!AF43,"2º do Grupo G")</f>
         <v>Egito</v>
       </c>
       <c r="L20" s="136" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>emp</v>
       </c>
       <c r="M20" s="133" t="str">
         <f>IF(OR(G20="",I20=""),"Vencedor 88",IF(G20&lt;&gt;I20,IF(G20&gt;I20,E20,K20),IF(SUM(F20:G20)=SUM(I20:J20),"Vencedor 88",IF(SUM(F20:G20)&gt;SUM(I20:J20),E20,K20))))</f>
-        <v>Vencedor 88</v>
+        <v>Egito</v>
       </c>
       <c r="N20" s="133">
         <v>88</v>
@@ -56494,11 +56522,15 @@
         <v>Paraguai</v>
       </c>
       <c r="F25" s="149"/>
-      <c r="G25" s="123"/>
+      <c r="G25" s="123">
+        <v>0</v>
+      </c>
       <c r="H25" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I25" s="123"/>
+      <c r="I25" s="123">
+        <v>1</v>
+      </c>
       <c r="J25" s="150"/>
       <c r="K25" s="151" t="str">
         <f>M9</f>
@@ -56510,7 +56542,7 @@
       </c>
       <c r="M25" s="133" t="str">
         <f>IF(OR(G25="",I25=""),"Vencedor 89",IF(G25&lt;&gt;I25,IF(G25&gt;I25,E25,K25),IF(SUM(F25:G25)=SUM(I25:J25),"Vencedor 89",IF(SUM(F25:G25)&gt;SUM(I25:J25),E25,K25))))</f>
-        <v>Vencedor 89</v>
+        <v>França</v>
       </c>
       <c r="N25" s="133">
         <v>89</v>
@@ -56572,11 +56604,15 @@
         <v>Canadá</v>
       </c>
       <c r="F26" s="149"/>
-      <c r="G26" s="123"/>
+      <c r="G26" s="123">
+        <v>0</v>
+      </c>
       <c r="H26" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I26" s="123"/>
+      <c r="I26" s="123">
+        <v>3</v>
+      </c>
       <c r="J26" s="150"/>
       <c r="K26" s="151" t="str">
         <f>M7</f>
@@ -56588,7 +56624,7 @@
       </c>
       <c r="M26" s="133" t="str">
         <f>IF(OR(G26="",I26=""),"Vencedor 90",IF(G26&lt;&gt;I26,IF(G26&gt;I26,E26,K26),IF(SUM(F26:G26)=SUM(I26:J26),"Vencedor 90",IF(SUM(F26:G26)&gt;SUM(I26:J26),E26,K26))))</f>
-        <v>Vencedor 90</v>
+        <v>Marrocos</v>
       </c>
       <c r="N26" s="133">
         <v>90</v>
@@ -56616,11 +56652,15 @@
         <v>Brasil</v>
       </c>
       <c r="F27" s="149"/>
-      <c r="G27" s="123"/>
+      <c r="G27" s="123">
+        <v>1</v>
+      </c>
       <c r="H27" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="123"/>
+      <c r="I27" s="123">
+        <v>2</v>
+      </c>
       <c r="J27" s="150"/>
       <c r="K27" s="151" t="str">
         <f>M10</f>
@@ -56632,7 +56672,7 @@
       </c>
       <c r="M27" s="133" t="str">
         <f>IF(OR(G27="",I27=""),"Vencedor 91",IF(G27&lt;&gt;I27,IF(G27&gt;I27,E27,K27),IF(SUM(F27:G27)=SUM(I27:J27),"Vencedor 91",IF(SUM(F27:G27)&gt;SUM(I27:J27),E27,K27))))</f>
-        <v>Vencedor 91</v>
+        <v>Noruega</v>
       </c>
       <c r="N27" s="133">
         <v>91</v>
@@ -56660,11 +56700,15 @@
         <v>México</v>
       </c>
       <c r="F28" s="149"/>
-      <c r="G28" s="123"/>
+      <c r="G28" s="123">
+        <v>2</v>
+      </c>
       <c r="H28" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="123"/>
+      <c r="I28" s="123">
+        <v>3</v>
+      </c>
       <c r="J28" s="150"/>
       <c r="K28" s="151" t="str">
         <f>M12</f>
@@ -56676,7 +56720,7 @@
       </c>
       <c r="M28" s="133" t="str">
         <f>IF(OR(G28="",I28=""),"Vencedor 92",IF(G28&lt;&gt;I28,IF(G28&gt;I28,E28,K28),IF(SUM(F28:G28)=SUM(I28:J28),"Vencedor 92",IF(SUM(F28:G28)&gt;SUM(I28:J28),E28,K28))))</f>
-        <v>Vencedor 92</v>
+        <v>Inglaterra</v>
       </c>
       <c r="N28" s="133">
         <v>92</v>
@@ -56707,7 +56751,7 @@
       </c>
       <c r="E29" s="106" t="str">
         <f>M15</f>
-        <v>Vencedor 83</v>
+        <v>Portugal</v>
       </c>
       <c r="F29" s="149"/>
       <c r="G29" s="123"/>
@@ -56718,7 +56762,7 @@
       <c r="J29" s="150"/>
       <c r="K29" s="151" t="str">
         <f>M16</f>
-        <v>Vencedor 84</v>
+        <v>Espanha</v>
       </c>
       <c r="L29" s="136" t="str">
         <f t="shared" si="18"/>
@@ -56803,7 +56847,7 @@
       </c>
       <c r="E31" s="106" t="str">
         <f>M18</f>
-        <v>Vencedor 86</v>
+        <v>Argentina</v>
       </c>
       <c r="F31" s="149"/>
       <c r="G31" s="123"/>
@@ -56814,7 +56858,7 @@
       <c r="J31" s="150"/>
       <c r="K31" s="151" t="str">
         <f>M20</f>
-        <v>Vencedor 88</v>
+        <v>Egito</v>
       </c>
       <c r="L31" s="136" t="str">
         <f t="shared" si="18"/>
@@ -56851,7 +56895,7 @@
       </c>
       <c r="E32" s="106" t="str">
         <f>M17</f>
-        <v>Vencedor 85</v>
+        <v>Suiça</v>
       </c>
       <c r="F32" s="149"/>
       <c r="G32" s="123"/>
@@ -57097,23 +57141,8 @@
       <c r="K82" s="45"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="8JRv5B/B5jMSXJQTg3Gidv52YDGKsjKvo30SeOBaK6JSNYAMZQ/wPbZnASuXj0gcQnaFpGbQs8ZzG0RfUFK9kg==" saltValue="BbqaqtGKXaW/tQWh+QEg4w==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="vyOy7e+Kipl/iIim/AhmV04T3MRdO7XqZOrn9PPXS3pWOghvTWOXD8HUj7i1Pq8tpKgw5m5Lutctpe8ebuImew==" saltValue="GsBJjoEg17jBuxUGR0mlBg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="31">
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AB34:AG34"/>
-    <mergeCell ref="AB35:AG35"/>
-    <mergeCell ref="AB36:AG36"/>
-    <mergeCell ref="B23:K23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="Y35:AA35"/>
-    <mergeCell ref="Y36:AA36"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AE24"/>
-    <mergeCell ref="AF24:AG24"/>
-    <mergeCell ref="Y34:AA34"/>
-    <mergeCell ref="AD28:AG28"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:I4"/>
@@ -57130,6 +57159,21 @@
     <mergeCell ref="AF18:AG18"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="AC4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AB34:AG34"/>
+    <mergeCell ref="AB35:AG35"/>
+    <mergeCell ref="AB36:AG36"/>
+    <mergeCell ref="B23:K23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="Y35:AA35"/>
+    <mergeCell ref="Y36:AA36"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AE24"/>
+    <mergeCell ref="AF24:AG24"/>
+    <mergeCell ref="Y34:AA34"/>
+    <mergeCell ref="AD28:AG28"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A2 B2:K2 X9:AG10 X15:AG16 X20:AG21 B21:K22 AB34:AB36 A57:K58 H59:K61 B62:K71 B83:K1048576">
     <cfRule type="cellIs" dxfId="27" priority="76" operator="equal">
@@ -57892,12 +57936,6 @@
     <sortCondition ref="C59:C64"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="N4:N6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="J4:J6"/>
-    <mergeCell ref="L4:L6"/>
     <mergeCell ref="AB4:AB6"/>
     <mergeCell ref="AD4:AD6"/>
     <mergeCell ref="AF4:AF6"/>
@@ -57908,6 +57946,12 @@
     <mergeCell ref="V4:V6"/>
     <mergeCell ref="X4:X6"/>
     <mergeCell ref="Z4:Z6"/>
+    <mergeCell ref="N4:N6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="J4:J6"/>
+    <mergeCell ref="L4:L6"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -58143,20 +58187,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -58179,14 +58223,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83E7837-68AD-48B2-A1AB-AAB452317AF5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="dc8c2798-6aba-4af7-93a4-b89253b03650"/>
@@ -58201,4 +58237,12 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Att Oitavas Dia 3
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED78202-39B0-4377-A87D-8EDFD748F56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C004B20-35B6-49E6-8924-68E165489957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
@@ -55205,7 +55205,7 @@
       </c>
       <c r="AA6" s="106" t="str">
         <f>M29</f>
-        <v>Vencedor 93</v>
+        <v>Espanha</v>
       </c>
       <c r="AB6" s="149"/>
       <c r="AC6" s="123"/>
@@ -55216,7 +55216,7 @@
       <c r="AF6" s="150"/>
       <c r="AG6" s="151" t="str">
         <f>M30</f>
-        <v>Vencedor 94</v>
+        <v>Bélgica</v>
       </c>
       <c r="AH6" s="136" t="str">
         <f t="shared" ref="AH6:AH8" si="1">IF(OR(AC6="",AE6=""),"",IF(AC6=AE6,"emp",""))</f>
@@ -56227,7 +56227,7 @@
         <v>22</v>
       </c>
       <c r="I19" s="123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" s="150"/>
       <c r="K19" s="151" t="str">
@@ -56236,11 +56236,11 @@
       </c>
       <c r="L19" s="136" t="str">
         <f t="shared" si="4"/>
-        <v>emp</v>
+        <v/>
       </c>
       <c r="M19" s="133" t="str">
         <f>IF(OR(G19="",I19=""),"Vencedor 87",IF(G19&lt;&gt;I19,IF(G19&gt;I19,E19,K19),IF(SUM(F19:G19)=SUM(I19:J19),"Vencedor 87",IF(SUM(F19:G19)&gt;SUM(I19:J19),E19,K19))))</f>
-        <v>Vencedor 87</v>
+        <v>Colômbia</v>
       </c>
       <c r="N19" s="133">
         <v>87</v>
@@ -56754,11 +56754,15 @@
         <v>Portugal</v>
       </c>
       <c r="F29" s="149"/>
-      <c r="G29" s="123"/>
+      <c r="G29" s="123">
+        <v>0</v>
+      </c>
       <c r="H29" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I29" s="123"/>
+      <c r="I29" s="123">
+        <v>1</v>
+      </c>
       <c r="J29" s="150"/>
       <c r="K29" s="151" t="str">
         <f>M16</f>
@@ -56770,7 +56774,7 @@
       </c>
       <c r="M29" s="133" t="str">
         <f>IF(OR(G29="",I29=""),"Vencedor 93",IF(G29&lt;&gt;I29,IF(G29&gt;I29,E29,K29),IF(SUM(F29:G29)=SUM(I29:J29),"Vencedor 93",IF(SUM(F29:G29)&gt;SUM(I29:J29),E29,K29))))</f>
-        <v>Vencedor 93</v>
+        <v>Espanha</v>
       </c>
       <c r="N29" s="133">
         <v>93</v>
@@ -56802,11 +56806,15 @@
         <v>Estados Unidos</v>
       </c>
       <c r="F30" s="149"/>
-      <c r="G30" s="123"/>
+      <c r="G30" s="123">
+        <v>1</v>
+      </c>
       <c r="H30" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I30" s="123"/>
+      <c r="I30" s="123">
+        <v>4</v>
+      </c>
       <c r="J30" s="150"/>
       <c r="K30" s="151" t="str">
         <f>M14</f>
@@ -56818,7 +56826,7 @@
       </c>
       <c r="M30" s="133" t="str">
         <f>IF(OR(G30="",I30=""),"Vencedor 94",IF(G30&lt;&gt;I30,IF(G30&gt;I30,E30,K30),IF(SUM(F30:G30)=SUM(I30:J30),"Vencedor 94",IF(SUM(F30:G30)&gt;SUM(I30:J30),E30,K30))))</f>
-        <v>Vencedor 94</v>
+        <v>Bélgica</v>
       </c>
       <c r="N30" s="133">
         <v>94</v>
@@ -56906,7 +56914,7 @@
       <c r="J32" s="150"/>
       <c r="K32" s="151" t="str">
         <f>M19</f>
-        <v>Vencedor 87</v>
+        <v>Colômbia</v>
       </c>
       <c r="L32" s="136" t="str">
         <f t="shared" si="18"/>
@@ -57143,6 +57151,21 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="vyOy7e+Kipl/iIim/AhmV04T3MRdO7XqZOrn9PPXS3pWOghvTWOXD8HUj7i1Pq8tpKgw5m5Lutctpe8ebuImew==" saltValue="GsBJjoEg17jBuxUGR0mlBg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="31">
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AB34:AG34"/>
+    <mergeCell ref="AB35:AG35"/>
+    <mergeCell ref="AB36:AG36"/>
+    <mergeCell ref="B23:K23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="Y35:AA35"/>
+    <mergeCell ref="Y36:AA36"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AE24"/>
+    <mergeCell ref="AF24:AG24"/>
+    <mergeCell ref="Y34:AA34"/>
+    <mergeCell ref="AD28:AG28"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:I4"/>
@@ -57159,21 +57182,6 @@
     <mergeCell ref="AF18:AG18"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="AC4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AB34:AG34"/>
-    <mergeCell ref="AB35:AG35"/>
-    <mergeCell ref="AB36:AG36"/>
-    <mergeCell ref="B23:K23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="Y35:AA35"/>
-    <mergeCell ref="Y36:AA36"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AE24"/>
-    <mergeCell ref="AF24:AG24"/>
-    <mergeCell ref="Y34:AA34"/>
-    <mergeCell ref="AD28:AG28"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A2 B2:K2 X9:AG10 X15:AG16 X20:AG21 B21:K22 AB34:AB36 A57:K58 H59:K61 B62:K71 B83:K1048576">
     <cfRule type="cellIs" dxfId="27" priority="76" operator="equal">
@@ -57936,6 +57944,12 @@
     <sortCondition ref="C59:C64"/>
   </sortState>
   <mergeCells count="16">
+    <mergeCell ref="N4:N6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="J4:J6"/>
+    <mergeCell ref="L4:L6"/>
     <mergeCell ref="AB4:AB6"/>
     <mergeCell ref="AD4:AD6"/>
     <mergeCell ref="AF4:AF6"/>
@@ -57946,12 +57960,6 @@
     <mergeCell ref="V4:V6"/>
     <mergeCell ref="X4:X6"/>
     <mergeCell ref="Z4:Z6"/>
-    <mergeCell ref="N4:N6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="J4:J6"/>
-    <mergeCell ref="L4:L6"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -58187,20 +58195,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -58223,6 +58231,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83E7837-68AD-48B2-A1AB-AAB452317AF5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="dc8c2798-6aba-4af7-93a4-b89253b03650"/>
@@ -58237,12 +58253,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Att Quartas de Final Completa
</commit_message>
<xml_diff>
--- a/Copa do Mundo FIFA 2026.xlsx
+++ b/Copa do Mundo FIFA 2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C004B20-35B6-49E6-8924-68E165489957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14BCC7B-B706-4F61-ABEE-DBA77B085FD5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="BcI4NY5Ohir363+nRCln2YCzlnOeJyINjZ1aV0hb2IpPHmsHZPUFroFzrod6xokqyCn7GUW2N1Z+U/w2mbyNbQ==" workbookSaltValue="VvXyFesAZC8L8IOzNm6PtA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9525" activeTab="5" xr2:uid="{076F3B28-812E-4458-A424-96085A053123}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="7" r:id="rId1"/>
@@ -26,17 +26,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -3009,17 +2998,6 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -3124,6 +3102,17 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -9428,25 +9417,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CB5EB0A-66D8-48B4-BC40-E2D214AFC03A}" name="Tabela1" displayName="Tabela1" ref="C3:E51" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9CB5EB0A-66D8-48B4-BC40-E2D214AFC03A}" name="Tabela1" displayName="Tabela1" ref="C3:E51" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
   <autoFilter ref="C3:E51" xr:uid="{9CB5EB0A-66D8-48B4-BC40-E2D214AFC03A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{BA403FB9-D643-4201-89E9-82280DBD496D}" name=" " dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{8927B163-5C71-4390-8413-1CB7AFCDC479}" name="Times" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{95E8A229-CD3E-4FE0-BC0B-3E68BBDC2143}" name="  " dataDxfId="86"/>
+    <tableColumn id="1" xr3:uid="{BA403FB9-D643-4201-89E9-82280DBD496D}" name=" " dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{8927B163-5C71-4390-8413-1CB7AFCDC479}" name="Times" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{95E8A229-CD3E-4FE0-BC0B-3E68BBDC2143}" name="  " dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -9484,7 +9473,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -9590,7 +9579,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -9732,7 +9721,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -10041,12 +10030,12 @@
     <mergeCell ref="J33:L33"/>
   </mergeCells>
   <conditionalFormatting sqref="J31:L31 J32:J33">
-    <cfRule type="cellIs" dxfId="85" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="2" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J31:L33">
-    <cfRule type="expression" dxfId="84" priority="1">
+    <cfRule type="expression" dxfId="89" priority="1">
       <formula>M31&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
@@ -55122,11 +55111,15 @@
         <v>França</v>
       </c>
       <c r="AB5" s="149"/>
-      <c r="AC5" s="123"/>
+      <c r="AC5" s="123">
+        <v>2</v>
+      </c>
       <c r="AD5" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="AE5" s="123"/>
+      <c r="AE5" s="123">
+        <v>0</v>
+      </c>
       <c r="AF5" s="150"/>
       <c r="AG5" s="151" t="str">
         <f>M26</f>
@@ -55138,7 +55131,7 @@
       </c>
       <c r="AI5" s="133" t="str">
         <f>IF(OR(AC5="",AE5=""),"Vencedor Q1",IF(AC5&lt;&gt;AE5,IF(AC5&gt;AE5,AA5,AG5),IF(SUM(AB5:AC5)=SUM(AE5:AF5),"Vencedor Q1",IF(SUM(AB5:AC5)&gt;SUM(AE5:AF5),AA5,AG5))))</f>
-        <v>Vencedor Q1</v>
+        <v>França</v>
       </c>
       <c r="AJ5" s="133"/>
       <c r="AK5" s="133"/>
@@ -55208,11 +55201,15 @@
         <v>Espanha</v>
       </c>
       <c r="AB6" s="149"/>
-      <c r="AC6" s="123"/>
+      <c r="AC6" s="123">
+        <v>2</v>
+      </c>
       <c r="AD6" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="AE6" s="123"/>
+      <c r="AE6" s="123">
+        <v>1</v>
+      </c>
       <c r="AF6" s="150"/>
       <c r="AG6" s="151" t="str">
         <f>M30</f>
@@ -55224,7 +55221,7 @@
       </c>
       <c r="AI6" s="133" t="str">
         <f>IF(OR(AC6="",AE6=""),"Vencedor Q2",IF(AC6&lt;&gt;AE6,IF(AC6&gt;AE6,AA6,AG6),IF(SUM(AB6:AC6)=SUM(AE6:AF6),"Vencedor Q2",IF(SUM(AB6:AC6)&gt;SUM(AE6:AF6),AA6,AG6))))</f>
-        <v>Vencedor Q2</v>
+        <v>Espanha</v>
       </c>
       <c r="AJ6" s="133"/>
       <c r="AK6" s="133"/>
@@ -55290,11 +55287,15 @@
         <v>Noruega</v>
       </c>
       <c r="AB7" s="149"/>
-      <c r="AC7" s="123"/>
+      <c r="AC7" s="123">
+        <v>1</v>
+      </c>
       <c r="AD7" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="AE7" s="123"/>
+      <c r="AE7" s="123">
+        <v>2</v>
+      </c>
       <c r="AF7" s="150"/>
       <c r="AG7" s="151" t="str">
         <f>M28</f>
@@ -55306,7 +55307,7 @@
       </c>
       <c r="AI7" s="133" t="str">
         <f>IF(OR(AC7="",AE7=""),"Vencedor Q3",IF(AC7&lt;&gt;AE7,IF(AC7&gt;AE7,AA7,AG7),IF(SUM(AB7:AC7)=SUM(AE7:AF7),"Vencedor Q3",IF(SUM(AB7:AC7)&gt;SUM(AE7:AF7),AA7,AG7))))</f>
-        <v>Vencedor Q3</v>
+        <v>Inglaterra</v>
       </c>
       <c r="AJ7" s="133"/>
       <c r="AK7" s="133"/>
@@ -55382,18 +55383,22 @@
       </c>
       <c r="AA8" s="106" t="str">
         <f>M31</f>
-        <v>Vencedor 95</v>
+        <v>Argentina</v>
       </c>
       <c r="AB8" s="149"/>
-      <c r="AC8" s="123"/>
+      <c r="AC8" s="123">
+        <v>3</v>
+      </c>
       <c r="AD8" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="AE8" s="123"/>
+      <c r="AE8" s="123">
+        <v>1</v>
+      </c>
       <c r="AF8" s="150"/>
       <c r="AG8" s="151" t="str">
         <f>M32</f>
-        <v>Vencedor 96</v>
+        <v>Suiça</v>
       </c>
       <c r="AH8" s="136" t="str">
         <f t="shared" si="1"/>
@@ -55401,7 +55406,7 @@
       </c>
       <c r="AI8" s="133" t="str">
         <f>IF(OR(AC8="",AE8=""),"Vencedor Q4",IF(AC8&lt;&gt;AE8,IF(AC8&gt;AE8,AA8,AG8),IF(SUM(AB8:AC8)=SUM(AE8:AF8),"Vencedor Q4",IF(SUM(AB8:AC8)&gt;SUM(AE8:AF8),AA8,AG8))))</f>
-        <v>Vencedor Q4</v>
+        <v>Argentina</v>
       </c>
       <c r="AJ8" s="133"/>
       <c r="AK8" s="133"/>
@@ -55794,7 +55799,7 @@
       </c>
       <c r="AA13" s="106" t="str">
         <f>AI5</f>
-        <v>Vencedor Q1</v>
+        <v>França</v>
       </c>
       <c r="AB13" s="149"/>
       <c r="AC13" s="123"/>
@@ -55805,7 +55810,7 @@
       <c r="AF13" s="150"/>
       <c r="AG13" s="151" t="str">
         <f>AI6</f>
-        <v>Vencedor Q2</v>
+        <v>Espanha</v>
       </c>
       <c r="AH13" s="136" t="str">
         <f>IF(OR(AC13="",AE13=""),"",IF(AC13=AE13,"emp",""))</f>
@@ -55890,7 +55895,7 @@
       </c>
       <c r="AA14" s="106" t="str">
         <f>AI7</f>
-        <v>Vencedor Q3</v>
+        <v>Inglaterra</v>
       </c>
       <c r="AB14" s="149"/>
       <c r="AC14" s="123"/>
@@ -55901,7 +55906,7 @@
       <c r="AF14" s="150"/>
       <c r="AG14" s="151" t="str">
         <f>AI8</f>
-        <v>Vencedor Q4</v>
+        <v>Argentina</v>
       </c>
       <c r="AH14" s="136" t="str">
         <f t="shared" ref="AH14" si="6">IF(OR(AC14="",AE14=""),"",IF(AC14=AE14,"emp",""))</f>
@@ -56858,11 +56863,15 @@
         <v>Argentina</v>
       </c>
       <c r="F31" s="149"/>
-      <c r="G31" s="123"/>
+      <c r="G31" s="123">
+        <v>3</v>
+      </c>
       <c r="H31" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I31" s="123"/>
+      <c r="I31" s="123">
+        <v>2</v>
+      </c>
       <c r="J31" s="150"/>
       <c r="K31" s="151" t="str">
         <f>M20</f>
@@ -56874,7 +56883,7 @@
       </c>
       <c r="M31" s="133" t="str">
         <f>IF(OR(G31="",I31=""),"Vencedor 95",IF(G31&lt;&gt;I31,IF(G31&gt;I31,E31,K31),IF(SUM(F31:G31)=SUM(I31:J31),"Vencedor 95",IF(SUM(F31:G31)&gt;SUM(I31:J31),E31,K31))))</f>
-        <v>Vencedor 95</v>
+        <v>Argentina</v>
       </c>
       <c r="N31" s="133">
         <v>95</v>
@@ -56905,24 +56914,32 @@
         <f>M17</f>
         <v>Suiça</v>
       </c>
-      <c r="F32" s="149"/>
-      <c r="G32" s="123"/>
+      <c r="F32" s="149">
+        <v>4</v>
+      </c>
+      <c r="G32" s="123">
+        <v>0</v>
+      </c>
       <c r="H32" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="I32" s="123"/>
-      <c r="J32" s="150"/>
+      <c r="I32" s="123">
+        <v>0</v>
+      </c>
+      <c r="J32" s="150">
+        <v>3</v>
+      </c>
       <c r="K32" s="151" t="str">
         <f>M19</f>
         <v>Colômbia</v>
       </c>
       <c r="L32" s="136" t="str">
         <f t="shared" si="18"/>
-        <v/>
+        <v>emp</v>
       </c>
       <c r="M32" s="133" t="str">
         <f>IF(OR(G32="",I32=""),"Vencedor 96",IF(G32&lt;&gt;I32,IF(G32&gt;I32,E32,K32),IF(SUM(F32:G32)=SUM(I32:J32),"Vencedor 96",IF(SUM(F32:G32)&gt;SUM(I32:J32),E32,K32))))</f>
-        <v>Vencedor 96</v>
+        <v>Suiça</v>
       </c>
       <c r="N32" s="133">
         <v>96</v>
@@ -57151,21 +57168,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="vyOy7e+Kipl/iIim/AhmV04T3MRdO7XqZOrn9PPXS3pWOghvTWOXD8HUj7i1Pq8tpKgw5m5Lutctpe8ebuImew==" saltValue="GsBJjoEg17jBuxUGR0mlBg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="31">
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AB34:AG34"/>
-    <mergeCell ref="AB35:AG35"/>
-    <mergeCell ref="AB36:AG36"/>
-    <mergeCell ref="B23:K23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="Y35:AA35"/>
-    <mergeCell ref="Y36:AA36"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AE24"/>
-    <mergeCell ref="AF24:AG24"/>
-    <mergeCell ref="Y34:AA34"/>
-    <mergeCell ref="AD28:AG28"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:I4"/>
@@ -57182,6 +57184,21 @@
     <mergeCell ref="AF18:AG18"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="AC4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AB34:AG34"/>
+    <mergeCell ref="AB35:AG35"/>
+    <mergeCell ref="AB36:AG36"/>
+    <mergeCell ref="B23:K23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="Y35:AA35"/>
+    <mergeCell ref="Y36:AA36"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AE24"/>
+    <mergeCell ref="AF24:AG24"/>
+    <mergeCell ref="Y34:AA34"/>
+    <mergeCell ref="AD28:AG28"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A2 B2:K2 X9:AG10 X15:AG16 X20:AG21 B21:K22 AB34:AB36 A57:K58 H59:K61 B62:K71 B83:K1048576">
     <cfRule type="cellIs" dxfId="27" priority="76" operator="equal">
@@ -57940,16 +57957,10 @@
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="c6tPJJQuMaLYYVxDkvgugaxcC+Uv5gkJkUqZgIt2uuxbzexMxqxVyEOkWorUUitpEJ1MPNBlUf/aYq65/wymIg==" saltValue="0J8NZQ0DnJYkRWhoKBlPHA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C59:C64">
+  <sortState ref="C59:C64">
     <sortCondition ref="C59:C64"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="N4:N6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="J4:J6"/>
-    <mergeCell ref="L4:L6"/>
     <mergeCell ref="AB4:AB6"/>
     <mergeCell ref="AD4:AD6"/>
     <mergeCell ref="AF4:AF6"/>
@@ -57960,6 +57971,12 @@
     <mergeCell ref="V4:V6"/>
     <mergeCell ref="X4:X6"/>
     <mergeCell ref="Z4:Z6"/>
+    <mergeCell ref="N4:N6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="J4:J6"/>
+    <mergeCell ref="L4:L6"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -57968,6 +57985,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DBF2846C41E31A469E3CED25F2422E48" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5fe40c83f7497f6a132ba44389c75f2c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2c8c20e6-817c-474f-b9c2-eb2b1ac24837" xmlns:ns4="dc8c2798-6aba-4af7-93a4-b89253b03650" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7827a91f6681aa3909757bf20cf55ac7" ns3:_="" ns4:_="">
     <xsd:import namespace="2c8c20e6-817c-474f-b9c2-eb2b1ac24837"/>
@@ -58194,24 +58228,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83E7837-68AD-48B2-A1AB-AAB452317AF5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="dc8c2798-6aba-4af7-93a4-b89253b03650"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2c8c20e6-817c-474f-b9c2-eb2b1ac24837"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dc8c2798-6aba-4af7-93a4-b89253b03650" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E4CC2DB-337D-464E-B291-77CE670D3A8E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58228,29 +58270,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45D7D45-1E18-48AE-827B-096C3C02C976}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83E7837-68AD-48B2-A1AB-AAB452317AF5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="dc8c2798-6aba-4af7-93a4-b89253b03650"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2c8c20e6-817c-474f-b9c2-eb2b1ac24837"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>